<commit_message>
Keep both El Hadji NTFP scenarios (biochar and revised).
Restore the original biochar workbook with all six methods and add a companion file with only the three revised NTFP rows, giving nine El Hadji models in the dashboard and master database (183 total).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Consultants Data Validation - Master Database.xlsx
+++ b/Consultants Data Validation - Master Database.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:HW181"/>
+  <dimension ref="A1:HW184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50366,7 +50366,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
+          <t>Southern Mauritania Afforestation - Date Palm with Biochar</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -50729,7 +50729,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
+          <t>Southern Mauritania Afforestation - Date Palm with Biochar</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -50760,25 +50760,25 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Seed Dispersal</t>
+          <t>ANR/50% Enrichment (NTFP)</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>seed_dispersal</t>
+          <t>anr_30_ntfp</t>
         </is>
       </c>
       <c r="J170" t="n">
-        <v>4965</v>
+        <v>6978</v>
       </c>
       <c r="K170" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="L170" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="M170" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N170" t="n">
         <v>2</v>
@@ -50787,7 +50787,7 @@
         <v>20</v>
       </c>
       <c r="P170" t="n">
-        <v>389</v>
+        <v>400</v>
       </c>
       <c r="Q170" t="inlineStr"/>
       <c r="R170" t="inlineStr"/>
@@ -50816,15 +50816,33 @@
       <c r="AO170" t="inlineStr"/>
       <c r="AP170" t="inlineStr"/>
       <c r="AQ170" t="inlineStr"/>
-      <c r="AR170" t="inlineStr"/>
-      <c r="AS170" t="inlineStr"/>
-      <c r="AT170" t="inlineStr"/>
-      <c r="AU170" t="inlineStr"/>
-      <c r="AV170" t="inlineStr"/>
-      <c r="AW170" t="inlineStr"/>
-      <c r="AX170" t="inlineStr"/>
-      <c r="AY170" t="inlineStr"/>
-      <c r="AZ170" t="inlineStr"/>
+      <c r="AR170" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS170" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT170" t="n">
+        <v>360</v>
+      </c>
+      <c r="AU170" t="n">
+        <v>7</v>
+      </c>
+      <c r="AV170" t="n">
+        <v>10</v>
+      </c>
+      <c r="AW170" t="n">
+        <v>570</v>
+      </c>
+      <c r="AX170" t="n">
+        <v>11</v>
+      </c>
+      <c r="AY170" t="n">
+        <v>20</v>
+      </c>
+      <c r="AZ170" t="n">
+        <v>820</v>
+      </c>
       <c r="BA170" t="inlineStr"/>
       <c r="BB170" t="inlineStr"/>
       <c r="BC170" t="inlineStr"/>
@@ -50846,12 +50864,24 @@
       <c r="BS170" t="inlineStr"/>
       <c r="BT170" t="inlineStr"/>
       <c r="BU170" t="inlineStr"/>
-      <c r="BV170" t="inlineStr"/>
-      <c r="BW170" t="inlineStr"/>
-      <c r="BX170" t="inlineStr"/>
-      <c r="BY170" t="inlineStr"/>
-      <c r="BZ170" t="inlineStr"/>
-      <c r="CA170" t="inlineStr"/>
+      <c r="BV170" t="n">
+        <v>7</v>
+      </c>
+      <c r="BW170" t="n">
+        <v>9</v>
+      </c>
+      <c r="BX170" t="n">
+        <v>480</v>
+      </c>
+      <c r="BY170" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ170" t="n">
+        <v>20</v>
+      </c>
+      <c r="CA170" t="n">
+        <v>550</v>
+      </c>
       <c r="CB170" t="inlineStr"/>
       <c r="CC170" t="inlineStr"/>
       <c r="CD170" t="inlineStr"/>
@@ -50883,7 +50913,7 @@
         <v>20</v>
       </c>
       <c r="DB170" t="n">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="DC170" t="inlineStr"/>
       <c r="DD170" t="inlineStr"/>
@@ -50919,7 +50949,7 @@
         <v>20</v>
       </c>
       <c r="EF170" t="n">
-        <v>139</v>
+        <v>185</v>
       </c>
       <c r="EG170" t="inlineStr"/>
       <c r="EH170" t="inlineStr"/>
@@ -50949,16 +50979,22 @@
       <c r="FF170" t="inlineStr"/>
       <c r="FG170" t="inlineStr"/>
       <c r="FH170" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="FI170" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="FJ170" t="n">
-        <v>8</v>
-      </c>
-      <c r="FK170" t="inlineStr"/>
-      <c r="FL170" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="FK170" t="inlineStr">
+        <is>
+          <t>Date palm Tree (Phoenix dactylifera) with Biochar</t>
+        </is>
+      </c>
+      <c r="FL170" t="n">
+        <v>2.89</v>
+      </c>
       <c r="FM170" t="inlineStr"/>
       <c r="FN170" t="inlineStr"/>
       <c r="FO170" t="inlineStr"/>
@@ -50974,15 +51010,33 @@
       <c r="FY170" t="inlineStr"/>
       <c r="FZ170" t="inlineStr"/>
       <c r="GA170" t="inlineStr"/>
-      <c r="GB170" t="inlineStr"/>
-      <c r="GC170" t="inlineStr"/>
-      <c r="GD170" t="inlineStr"/>
-      <c r="GE170" t="inlineStr"/>
-      <c r="GF170" t="inlineStr"/>
-      <c r="GG170" t="inlineStr"/>
-      <c r="GH170" t="inlineStr"/>
-      <c r="GI170" t="inlineStr"/>
-      <c r="GJ170" t="inlineStr"/>
+      <c r="GB170" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC170" t="n">
+        <v>6</v>
+      </c>
+      <c r="GD170" t="n">
+        <v>2700</v>
+      </c>
+      <c r="GE170" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF170" t="n">
+        <v>9</v>
+      </c>
+      <c r="GG170" t="n">
+        <v>14357</v>
+      </c>
+      <c r="GH170" t="n">
+        <v>10</v>
+      </c>
+      <c r="GI170" t="n">
+        <v>20</v>
+      </c>
+      <c r="GJ170" t="n">
+        <v>26479</v>
+      </c>
       <c r="GK170" t="inlineStr"/>
       <c r="GL170" t="inlineStr"/>
       <c r="GM170" t="inlineStr"/>
@@ -51092,7 +51146,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
+          <t>Southern Mauritania Afforestation - Date Palm with Biochar</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -51123,25 +51177,25 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Full Seedling Plantation</t>
+          <t>Seed Dispersal</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>seedling_planting</t>
+          <t>seed_dispersal</t>
         </is>
       </c>
       <c r="J171" t="n">
-        <v>7031</v>
+        <v>4965</v>
       </c>
       <c r="K171" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="L171" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="M171" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N171" t="n">
         <v>2</v>
@@ -51150,7 +51204,7 @@
         <v>20</v>
       </c>
       <c r="P171" t="n">
-        <v>461</v>
+        <v>389</v>
       </c>
       <c r="Q171" t="inlineStr"/>
       <c r="R171" t="inlineStr"/>
@@ -51246,7 +51300,7 @@
         <v>20</v>
       </c>
       <c r="DB171" t="n">
-        <v>221</v>
+        <v>145</v>
       </c>
       <c r="DC171" t="inlineStr"/>
       <c r="DD171" t="inlineStr"/>
@@ -51282,7 +51336,7 @@
         <v>20</v>
       </c>
       <c r="EF171" t="n">
-        <v>198</v>
+        <v>139</v>
       </c>
       <c r="EG171" t="inlineStr"/>
       <c r="EH171" t="inlineStr"/>
@@ -51312,13 +51366,13 @@
       <c r="FF171" t="inlineStr"/>
       <c r="FG171" t="inlineStr"/>
       <c r="FH171" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="FI171" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="FJ171" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="FK171" t="inlineStr"/>
       <c r="FL171" t="inlineStr"/>
@@ -51455,7 +51509,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
+          <t>Southern Mauritania Afforestation - Date Palm with Biochar</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -51486,29 +51540,35 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>ANR/50% Enrichment (NTFP)</t>
+          <t>Seed Dispersal (NTFP)</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>anr_30_ntfp</t>
+          <t>seed_dispersal_ntfp</t>
         </is>
       </c>
       <c r="J172" t="n">
-        <v>5678</v>
+        <v>8287</v>
       </c>
       <c r="K172" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="L172" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="M172" t="n">
-        <v>11</v>
-      </c>
-      <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr"/>
-      <c r="P172" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="N172" t="n">
+        <v>2</v>
+      </c>
+      <c r="O172" t="n">
+        <v>20</v>
+      </c>
+      <c r="P172" t="n">
+        <v>400</v>
+      </c>
       <c r="Q172" t="inlineStr"/>
       <c r="R172" t="inlineStr"/>
       <c r="S172" t="inlineStr"/>
@@ -51543,19 +51603,19 @@
         <v>6</v>
       </c>
       <c r="AT172" t="n">
-        <v>360</v>
+        <v>185</v>
       </c>
       <c r="AU172" t="n">
         <v>7</v>
       </c>
       <c r="AV172" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW172" t="n">
+        <v>390</v>
+      </c>
+      <c r="AX172" t="n">
         <v>10</v>
-      </c>
-      <c r="AW172" t="n">
-        <v>570</v>
-      </c>
-      <c r="AX172" t="n">
-        <v>11</v>
       </c>
       <c r="AY172" t="n">
         <v>20</v>
@@ -51585,13 +51645,13 @@
       <c r="BT172" t="inlineStr"/>
       <c r="BU172" t="inlineStr"/>
       <c r="BV172" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="BW172" t="n">
         <v>9</v>
       </c>
       <c r="BX172" t="n">
-        <v>480</v>
+        <v>245</v>
       </c>
       <c r="BY172" t="n">
         <v>10</v>
@@ -51633,7 +51693,7 @@
         <v>20</v>
       </c>
       <c r="DB172" t="n">
-        <v>205</v>
+        <v>119</v>
       </c>
       <c r="DC172" t="inlineStr"/>
       <c r="DD172" t="inlineStr"/>
@@ -51669,7 +51729,7 @@
         <v>20</v>
       </c>
       <c r="EF172" t="n">
-        <v>185</v>
+        <v>224</v>
       </c>
       <c r="EG172" t="inlineStr"/>
       <c r="EH172" t="inlineStr"/>
@@ -51709,7 +51769,7 @@
       </c>
       <c r="FK172" t="inlineStr">
         <is>
-          <t>Date palm Tree (Phoenix dactylifera)</t>
+          <t>Date palm Tree (Phoenix dactylifera) with Biochar</t>
         </is>
       </c>
       <c r="FL172" t="n">
@@ -51737,16 +51797,16 @@
         <v>6</v>
       </c>
       <c r="GD172" t="n">
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="GE172" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="GF172" t="n">
         <v>9</v>
       </c>
       <c r="GG172" t="n">
-        <v>11657</v>
+        <v>14685</v>
       </c>
       <c r="GH172" t="n">
         <v>10</v>
@@ -51755,7 +51815,7 @@
         <v>20</v>
       </c>
       <c r="GJ172" t="n">
-        <v>23779</v>
+        <v>26479</v>
       </c>
       <c r="GK172" t="inlineStr"/>
       <c r="GL172" t="inlineStr"/>
@@ -51866,7 +51926,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
+          <t>Southern Mauritania Afforestation - Date Palm with Biochar</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -51897,29 +51957,35 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Seed Dispersal (NTFP)</t>
+          <t>Full Seedling Plantation</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>seed_dispersal_ntfp</t>
+          <t>seedling_planting</t>
         </is>
       </c>
       <c r="J173" t="n">
-        <v>6987</v>
+        <v>7031</v>
       </c>
       <c r="K173" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="L173" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="M173" t="n">
-        <v>7</v>
-      </c>
-      <c r="N173" t="inlineStr"/>
-      <c r="O173" t="inlineStr"/>
-      <c r="P173" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="N173" t="n">
+        <v>2</v>
+      </c>
+      <c r="O173" t="n">
+        <v>20</v>
+      </c>
+      <c r="P173" t="n">
+        <v>461</v>
+      </c>
       <c r="Q173" t="inlineStr"/>
       <c r="R173" t="inlineStr"/>
       <c r="S173" t="inlineStr"/>
@@ -51947,33 +52013,15 @@
       <c r="AO173" t="inlineStr"/>
       <c r="AP173" t="inlineStr"/>
       <c r="AQ173" t="inlineStr"/>
-      <c r="AR173" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS173" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT173" t="n">
-        <v>185</v>
-      </c>
-      <c r="AU173" t="n">
-        <v>7</v>
-      </c>
-      <c r="AV173" t="n">
-        <v>9</v>
-      </c>
-      <c r="AW173" t="n">
-        <v>390</v>
-      </c>
-      <c r="AX173" t="n">
-        <v>10</v>
-      </c>
-      <c r="AY173" t="n">
-        <v>20</v>
-      </c>
-      <c r="AZ173" t="n">
-        <v>820</v>
-      </c>
+      <c r="AR173" t="inlineStr"/>
+      <c r="AS173" t="inlineStr"/>
+      <c r="AT173" t="inlineStr"/>
+      <c r="AU173" t="inlineStr"/>
+      <c r="AV173" t="inlineStr"/>
+      <c r="AW173" t="inlineStr"/>
+      <c r="AX173" t="inlineStr"/>
+      <c r="AY173" t="inlineStr"/>
+      <c r="AZ173" t="inlineStr"/>
       <c r="BA173" t="inlineStr"/>
       <c r="BB173" t="inlineStr"/>
       <c r="BC173" t="inlineStr"/>
@@ -51995,24 +52043,12 @@
       <c r="BS173" t="inlineStr"/>
       <c r="BT173" t="inlineStr"/>
       <c r="BU173" t="inlineStr"/>
-      <c r="BV173" t="n">
-        <v>6</v>
-      </c>
-      <c r="BW173" t="n">
-        <v>9</v>
-      </c>
-      <c r="BX173" t="n">
-        <v>245</v>
-      </c>
-      <c r="BY173" t="n">
-        <v>10</v>
-      </c>
-      <c r="BZ173" t="n">
-        <v>20</v>
-      </c>
-      <c r="CA173" t="n">
-        <v>550</v>
-      </c>
+      <c r="BV173" t="inlineStr"/>
+      <c r="BW173" t="inlineStr"/>
+      <c r="BX173" t="inlineStr"/>
+      <c r="BY173" t="inlineStr"/>
+      <c r="BZ173" t="inlineStr"/>
+      <c r="CA173" t="inlineStr"/>
       <c r="CB173" t="inlineStr"/>
       <c r="CC173" t="inlineStr"/>
       <c r="CD173" t="inlineStr"/>
@@ -52044,7 +52080,7 @@
         <v>20</v>
       </c>
       <c r="DB173" t="n">
-        <v>119</v>
+        <v>221</v>
       </c>
       <c r="DC173" t="inlineStr"/>
       <c r="DD173" t="inlineStr"/>
@@ -52080,7 +52116,7 @@
         <v>20</v>
       </c>
       <c r="EF173" t="n">
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="EG173" t="inlineStr"/>
       <c r="EH173" t="inlineStr"/>
@@ -52110,22 +52146,16 @@
       <c r="FF173" t="inlineStr"/>
       <c r="FG173" t="inlineStr"/>
       <c r="FH173" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="FI173" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="FJ173" t="n">
-        <v>9</v>
-      </c>
-      <c r="FK173" t="inlineStr">
-        <is>
-          <t>Date palm Tree (Phoenix dactylifera)</t>
-        </is>
-      </c>
-      <c r="FL173" t="n">
-        <v>2.89</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="FK173" t="inlineStr"/>
+      <c r="FL173" t="inlineStr"/>
       <c r="FM173" t="inlineStr"/>
       <c r="FN173" t="inlineStr"/>
       <c r="FO173" t="inlineStr"/>
@@ -52141,33 +52171,15 @@
       <c r="FY173" t="inlineStr"/>
       <c r="FZ173" t="inlineStr"/>
       <c r="GA173" t="inlineStr"/>
-      <c r="GB173" t="n">
-        <v>1</v>
-      </c>
-      <c r="GC173" t="n">
-        <v>6</v>
-      </c>
-      <c r="GD173" t="n">
-        <v>0</v>
-      </c>
-      <c r="GE173" t="n">
-        <v>7</v>
-      </c>
-      <c r="GF173" t="n">
-        <v>9</v>
-      </c>
-      <c r="GG173" t="n">
-        <v>11985</v>
-      </c>
-      <c r="GH173" t="n">
-        <v>10</v>
-      </c>
-      <c r="GI173" t="n">
-        <v>20</v>
-      </c>
-      <c r="GJ173" t="n">
-        <v>23779</v>
-      </c>
+      <c r="GB173" t="inlineStr"/>
+      <c r="GC173" t="inlineStr"/>
+      <c r="GD173" t="inlineStr"/>
+      <c r="GE173" t="inlineStr"/>
+      <c r="GF173" t="inlineStr"/>
+      <c r="GG173" t="inlineStr"/>
+      <c r="GH173" t="inlineStr"/>
+      <c r="GI173" t="inlineStr"/>
+      <c r="GJ173" t="inlineStr"/>
       <c r="GK173" t="inlineStr"/>
       <c r="GL173" t="inlineStr"/>
       <c r="GM173" t="inlineStr"/>
@@ -52277,7 +52289,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
+          <t>Southern Mauritania Afforestation - Date Palm with Biochar</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -52317,20 +52329,26 @@
         </is>
       </c>
       <c r="J174" t="n">
-        <v>8775</v>
+        <v>10075</v>
       </c>
       <c r="K174" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="L174" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="M174" t="n">
-        <v>13</v>
-      </c>
-      <c r="N174" t="inlineStr"/>
-      <c r="O174" t="inlineStr"/>
-      <c r="P174" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="N174" t="n">
+        <v>2</v>
+      </c>
+      <c r="O174" t="n">
+        <v>20</v>
+      </c>
+      <c r="P174" t="n">
+        <v>400</v>
+      </c>
       <c r="Q174" t="inlineStr"/>
       <c r="R174" t="inlineStr"/>
       <c r="S174" t="inlineStr"/>
@@ -52531,7 +52549,7 @@
       </c>
       <c r="FK174" t="inlineStr">
         <is>
-          <t>Date palm Tree (Phoenix dactylifera)</t>
+          <t>Date palm Tree (Phoenix dactylifera) with Biochar</t>
         </is>
       </c>
       <c r="FL174" t="n">
@@ -52559,7 +52577,7 @@
         <v>6</v>
       </c>
       <c r="GD174" t="n">
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="GE174" t="n">
         <v>7</v>
@@ -52568,7 +52586,7 @@
         <v>9</v>
       </c>
       <c r="GG174" t="n">
-        <v>13845</v>
+        <v>16545</v>
       </c>
       <c r="GH174" t="n">
         <v>10</v>
@@ -52577,7 +52595,7 @@
         <v>20</v>
       </c>
       <c r="GJ174" t="n">
-        <v>23779</v>
+        <v>26479</v>
       </c>
       <c r="GK174" t="inlineStr"/>
       <c r="GL174" t="inlineStr"/>
@@ -52688,70 +52706,60 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SAMUEL KIMENYI</t>
+          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>SAMUEL KIMENYI</t>
+          <t>El Hadji Beye</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>9720562.16, 753393.14</t>
-        </is>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Mountaine Forest</t>
+          <t>Arid or Semi-Arid Zones</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>Mauritania</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Kigali</t>
+          <t>Kaedi</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>ANR/50% Enrichment</t>
+          <t>ANR/50% Enrichment (NTFP)</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>anr_30</t>
+          <t>anr_30_ntfp</t>
         </is>
       </c>
       <c r="J175" t="n">
-        <v>651</v>
+        <v>5678</v>
       </c>
       <c r="K175" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L175" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M175" t="n">
-        <v>8</v>
-      </c>
-      <c r="N175" t="n">
-        <v>2</v>
-      </c>
-      <c r="O175" t="n">
-        <v>20</v>
-      </c>
-      <c r="P175" t="n">
-        <v>100</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
+      <c r="P175" t="inlineStr"/>
       <c r="Q175" t="inlineStr"/>
       <c r="R175" t="inlineStr"/>
       <c r="S175" t="inlineStr"/>
@@ -52779,15 +52787,33 @@
       <c r="AO175" t="inlineStr"/>
       <c r="AP175" t="inlineStr"/>
       <c r="AQ175" t="inlineStr"/>
-      <c r="AR175" t="inlineStr"/>
-      <c r="AS175" t="inlineStr"/>
-      <c r="AT175" t="inlineStr"/>
-      <c r="AU175" t="inlineStr"/>
-      <c r="AV175" t="inlineStr"/>
-      <c r="AW175" t="inlineStr"/>
-      <c r="AX175" t="inlineStr"/>
-      <c r="AY175" t="inlineStr"/>
-      <c r="AZ175" t="inlineStr"/>
+      <c r="AR175" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS175" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT175" t="n">
+        <v>360</v>
+      </c>
+      <c r="AU175" t="n">
+        <v>7</v>
+      </c>
+      <c r="AV175" t="n">
+        <v>10</v>
+      </c>
+      <c r="AW175" t="n">
+        <v>570</v>
+      </c>
+      <c r="AX175" t="n">
+        <v>11</v>
+      </c>
+      <c r="AY175" t="n">
+        <v>20</v>
+      </c>
+      <c r="AZ175" t="n">
+        <v>820</v>
+      </c>
       <c r="BA175" t="inlineStr"/>
       <c r="BB175" t="inlineStr"/>
       <c r="BC175" t="inlineStr"/>
@@ -52809,12 +52835,24 @@
       <c r="BS175" t="inlineStr"/>
       <c r="BT175" t="inlineStr"/>
       <c r="BU175" t="inlineStr"/>
-      <c r="BV175" t="inlineStr"/>
-      <c r="BW175" t="inlineStr"/>
-      <c r="BX175" t="inlineStr"/>
-      <c r="BY175" t="inlineStr"/>
-      <c r="BZ175" t="inlineStr"/>
-      <c r="CA175" t="inlineStr"/>
+      <c r="BV175" t="n">
+        <v>7</v>
+      </c>
+      <c r="BW175" t="n">
+        <v>9</v>
+      </c>
+      <c r="BX175" t="n">
+        <v>480</v>
+      </c>
+      <c r="BY175" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ175" t="n">
+        <v>20</v>
+      </c>
+      <c r="CA175" t="n">
+        <v>550</v>
+      </c>
       <c r="CB175" t="inlineStr"/>
       <c r="CC175" t="inlineStr"/>
       <c r="CD175" t="inlineStr"/>
@@ -52846,7 +52884,7 @@
         <v>20</v>
       </c>
       <c r="DB175" t="n">
-        <v>300</v>
+        <v>205</v>
       </c>
       <c r="DC175" t="inlineStr"/>
       <c r="DD175" t="inlineStr"/>
@@ -52882,7 +52920,7 @@
         <v>20</v>
       </c>
       <c r="EF175" t="n">
-        <v>220</v>
+        <v>185</v>
       </c>
       <c r="EG175" t="inlineStr"/>
       <c r="EH175" t="inlineStr"/>
@@ -52912,16 +52950,22 @@
       <c r="FF175" t="inlineStr"/>
       <c r="FG175" t="inlineStr"/>
       <c r="FH175" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="FI175" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="FJ175" t="n">
-        <v>22</v>
-      </c>
-      <c r="FK175" t="inlineStr"/>
-      <c r="FL175" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="FK175" t="inlineStr">
+        <is>
+          <t>Date palm Tree (Phoenix dactylifera)</t>
+        </is>
+      </c>
+      <c r="FL175" t="n">
+        <v>2.89</v>
+      </c>
       <c r="FM175" t="inlineStr"/>
       <c r="FN175" t="inlineStr"/>
       <c r="FO175" t="inlineStr"/>
@@ -52937,15 +52981,33 @@
       <c r="FY175" t="inlineStr"/>
       <c r="FZ175" t="inlineStr"/>
       <c r="GA175" t="inlineStr"/>
-      <c r="GB175" t="inlineStr"/>
-      <c r="GC175" t="inlineStr"/>
-      <c r="GD175" t="inlineStr"/>
-      <c r="GE175" t="inlineStr"/>
-      <c r="GF175" t="inlineStr"/>
-      <c r="GG175" t="inlineStr"/>
-      <c r="GH175" t="inlineStr"/>
-      <c r="GI175" t="inlineStr"/>
-      <c r="GJ175" t="inlineStr"/>
+      <c r="GB175" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC175" t="n">
+        <v>6</v>
+      </c>
+      <c r="GD175" t="n">
+        <v>0</v>
+      </c>
+      <c r="GE175" t="n">
+        <v>6</v>
+      </c>
+      <c r="GF175" t="n">
+        <v>9</v>
+      </c>
+      <c r="GG175" t="n">
+        <v>11657</v>
+      </c>
+      <c r="GH175" t="n">
+        <v>10</v>
+      </c>
+      <c r="GI175" t="n">
+        <v>20</v>
+      </c>
+      <c r="GJ175" t="n">
+        <v>23779</v>
+      </c>
       <c r="GK175" t="inlineStr"/>
       <c r="GL175" t="inlineStr"/>
       <c r="GM175" t="inlineStr"/>
@@ -52953,100 +53015,100 @@
       <c r="GO175" t="inlineStr"/>
       <c r="GP175" t="inlineStr"/>
       <c r="GQ175" t="n">
-        <v>3447.15</v>
+        <v>252.98</v>
       </c>
       <c r="GR175" t="n">
-        <v>975.001256306883</v>
+        <v>31.99972009877586</v>
       </c>
       <c r="GS175" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="GT175" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="GU175" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="GV175" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="GW175" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="GX175" t="n">
-        <v>4027.02</v>
+        <v>1000</v>
       </c>
       <c r="GY175" t="n">
-        <v>930.0004324128028</v>
+        <v>400</v>
       </c>
       <c r="GZ175" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="HA175" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="HB175" t="n">
+        <v>32</v>
+      </c>
+      <c r="HC175" t="n">
+        <v>9</v>
+      </c>
+      <c r="HD175" t="n">
+        <v>140</v>
+      </c>
+      <c r="HE175" t="n">
+        <v>10</v>
+      </c>
+      <c r="HF175" t="n">
+        <v>43</v>
+      </c>
+      <c r="HG175" t="n">
+        <v>43</v>
+      </c>
+      <c r="HH175" t="n">
+        <v>14</v>
+      </c>
+      <c r="HI175" t="n">
+        <v>116</v>
+      </c>
+      <c r="HJ175" t="n">
+        <v>15</v>
+      </c>
+      <c r="HK175" t="n">
+        <v>51</v>
+      </c>
+      <c r="HL175" t="n">
         <v>35</v>
       </c>
-      <c r="HC175" t="n">
-        <v>5</v>
-      </c>
-      <c r="HD175" t="n">
-        <v>150</v>
-      </c>
-      <c r="HE175" t="n">
-        <v>20</v>
-      </c>
-      <c r="HF175" t="n">
-        <v>72</v>
-      </c>
-      <c r="HG175" t="n">
-        <v>18</v>
-      </c>
-      <c r="HH175" t="n">
-        <v>10</v>
-      </c>
-      <c r="HI175" t="n">
+      <c r="HM175" t="n">
+        <v>14</v>
+      </c>
+      <c r="HN175" t="n">
         <v>100</v>
       </c>
-      <c r="HJ175" t="n">
-        <v>8</v>
-      </c>
-      <c r="HK175" t="n">
-        <v>60</v>
-      </c>
-      <c r="HL175" t="n">
-        <v>30</v>
-      </c>
-      <c r="HM175" t="n">
-        <v>10</v>
-      </c>
-      <c r="HN175" t="n">
-        <v>90</v>
-      </c>
       <c r="HO175" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="HP175" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="HQ175" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="HR175" t="n">
         <v>10</v>
       </c>
       <c r="HS175" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="HT175" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="HU175" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="HV175" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="HW175" t="n">
         <v>0</v>
@@ -53055,57 +53117,53 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SAMUEL KIMENYI</t>
+          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>SAMUEL KIMENYI</t>
+          <t>El Hadji Beye</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>9720562.16, 753393.14</t>
-        </is>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Mountaine Forest</t>
+          <t>Arid or Semi-Arid Zones</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>Mauritania</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Kigali</t>
+          <t>Kaedi</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>ANR/50% Enrichment (NTFP)</t>
+          <t>Seed Dispersal (NTFP)</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>anr_30_ntfp</t>
+          <t>seed_dispersal_ntfp</t>
         </is>
       </c>
       <c r="J176" t="n">
-        <v>785</v>
+        <v>6987</v>
       </c>
       <c r="K176" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="L176" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="M176" t="n">
         <v>7</v>
@@ -53144,17 +53202,29 @@
         <v>2</v>
       </c>
       <c r="AS176" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT176" t="n">
+        <v>185</v>
+      </c>
+      <c r="AU176" t="n">
+        <v>7</v>
+      </c>
+      <c r="AV176" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW176" t="n">
+        <v>390</v>
+      </c>
+      <c r="AX176" t="n">
+        <v>10</v>
+      </c>
+      <c r="AY176" t="n">
         <v>20</v>
       </c>
-      <c r="AT176" t="n">
-        <v>163</v>
-      </c>
-      <c r="AU176" t="inlineStr"/>
-      <c r="AV176" t="inlineStr"/>
-      <c r="AW176" t="inlineStr"/>
-      <c r="AX176" t="inlineStr"/>
-      <c r="AY176" t="inlineStr"/>
-      <c r="AZ176" t="inlineStr"/>
+      <c r="AZ176" t="n">
+        <v>820</v>
+      </c>
       <c r="BA176" t="inlineStr"/>
       <c r="BB176" t="inlineStr"/>
       <c r="BC176" t="inlineStr"/>
@@ -53177,17 +53247,23 @@
       <c r="BT176" t="inlineStr"/>
       <c r="BU176" t="inlineStr"/>
       <c r="BV176" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BW176" t="n">
+        <v>9</v>
+      </c>
+      <c r="BX176" t="n">
+        <v>245</v>
+      </c>
+      <c r="BY176" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ176" t="n">
         <v>20</v>
       </c>
-      <c r="BX176" t="n">
-        <v>150</v>
-      </c>
-      <c r="BY176" t="inlineStr"/>
-      <c r="BZ176" t="inlineStr"/>
-      <c r="CA176" t="inlineStr"/>
+      <c r="CA176" t="n">
+        <v>550</v>
+      </c>
       <c r="CB176" t="inlineStr"/>
       <c r="CC176" t="inlineStr"/>
       <c r="CD176" t="inlineStr"/>
@@ -53219,7 +53295,7 @@
         <v>20</v>
       </c>
       <c r="DB176" t="n">
-        <v>450</v>
+        <v>119</v>
       </c>
       <c r="DC176" t="inlineStr"/>
       <c r="DD176" t="inlineStr"/>
@@ -53255,7 +53331,7 @@
         <v>20</v>
       </c>
       <c r="EF176" t="n">
-        <v>390</v>
+        <v>224</v>
       </c>
       <c r="EG176" t="inlineStr"/>
       <c r="EH176" t="inlineStr"/>
@@ -53285,70 +53361,64 @@
       <c r="FF176" t="inlineStr"/>
       <c r="FG176" t="inlineStr"/>
       <c r="FH176" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="FI176" t="n">
         <v>22</v>
       </c>
       <c r="FJ176" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="FK176" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Yushania alpina</t>
+          <t>Date palm Tree (Phoenix dactylifera)</t>
         </is>
       </c>
       <c r="FL176" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="FM176" t="n">
-        <v>5</v>
-      </c>
-      <c r="FN176" t="n">
-        <v>9</v>
-      </c>
-      <c r="FO176" t="n">
-        <v>4100</v>
-      </c>
-      <c r="FP176" t="n">
-        <v>10</v>
-      </c>
-      <c r="FQ176" t="n">
-        <v>14</v>
-      </c>
-      <c r="FR176" t="n">
-        <v>8400</v>
-      </c>
-      <c r="FS176" t="n">
-        <v>15</v>
-      </c>
-      <c r="FT176" t="n">
-        <v>19</v>
-      </c>
-      <c r="FU176" t="n">
-        <v>11300</v>
-      </c>
-      <c r="FV176" t="n">
-        <v>20</v>
-      </c>
-      <c r="FW176" t="n">
-        <v>20</v>
-      </c>
-      <c r="FX176" t="n">
-        <v>13500</v>
-      </c>
+        <v>2.89</v>
+      </c>
+      <c r="FM176" t="inlineStr"/>
+      <c r="FN176" t="inlineStr"/>
+      <c r="FO176" t="inlineStr"/>
+      <c r="FP176" t="inlineStr"/>
+      <c r="FQ176" t="inlineStr"/>
+      <c r="FR176" t="inlineStr"/>
+      <c r="FS176" t="inlineStr"/>
+      <c r="FT176" t="inlineStr"/>
+      <c r="FU176" t="inlineStr"/>
+      <c r="FV176" t="inlineStr"/>
+      <c r="FW176" t="inlineStr"/>
+      <c r="FX176" t="inlineStr"/>
       <c r="FY176" t="inlineStr"/>
       <c r="FZ176" t="inlineStr"/>
       <c r="GA176" t="inlineStr"/>
-      <c r="GB176" t="inlineStr"/>
-      <c r="GC176" t="inlineStr"/>
-      <c r="GD176" t="inlineStr"/>
-      <c r="GE176" t="inlineStr"/>
-      <c r="GF176" t="inlineStr"/>
-      <c r="GG176" t="inlineStr"/>
-      <c r="GH176" t="inlineStr"/>
-      <c r="GI176" t="inlineStr"/>
-      <c r="GJ176" t="inlineStr"/>
+      <c r="GB176" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC176" t="n">
+        <v>6</v>
+      </c>
+      <c r="GD176" t="n">
+        <v>0</v>
+      </c>
+      <c r="GE176" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF176" t="n">
+        <v>9</v>
+      </c>
+      <c r="GG176" t="n">
+        <v>11985</v>
+      </c>
+      <c r="GH176" t="n">
+        <v>10</v>
+      </c>
+      <c r="GI176" t="n">
+        <v>20</v>
+      </c>
+      <c r="GJ176" t="n">
+        <v>23779</v>
+      </c>
       <c r="GK176" t="inlineStr"/>
       <c r="GL176" t="inlineStr"/>
       <c r="GM176" t="inlineStr"/>
@@ -53356,100 +53426,100 @@
       <c r="GO176" t="inlineStr"/>
       <c r="GP176" t="inlineStr"/>
       <c r="GQ176" t="n">
-        <v>3447.15</v>
+        <v>252.98</v>
       </c>
       <c r="GR176" t="n">
-        <v>975.001256306883</v>
+        <v>31.99972009877586</v>
       </c>
       <c r="GS176" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="GT176" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="GU176" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="GV176" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="GW176" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="GX176" t="n">
-        <v>4027.02</v>
+        <v>1000</v>
       </c>
       <c r="GY176" t="n">
-        <v>930.0004324128028</v>
+        <v>400</v>
       </c>
       <c r="GZ176" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="HA176" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="HB176" t="n">
+        <v>32</v>
+      </c>
+      <c r="HC176" t="n">
+        <v>9</v>
+      </c>
+      <c r="HD176" t="n">
+        <v>140</v>
+      </c>
+      <c r="HE176" t="n">
+        <v>10</v>
+      </c>
+      <c r="HF176" t="n">
+        <v>43</v>
+      </c>
+      <c r="HG176" t="n">
+        <v>43</v>
+      </c>
+      <c r="HH176" t="n">
+        <v>14</v>
+      </c>
+      <c r="HI176" t="n">
+        <v>116</v>
+      </c>
+      <c r="HJ176" t="n">
+        <v>15</v>
+      </c>
+      <c r="HK176" t="n">
+        <v>51</v>
+      </c>
+      <c r="HL176" t="n">
         <v>35</v>
       </c>
-      <c r="HC176" t="n">
-        <v>5</v>
-      </c>
-      <c r="HD176" t="n">
-        <v>150</v>
-      </c>
-      <c r="HE176" t="n">
-        <v>20</v>
-      </c>
-      <c r="HF176" t="n">
-        <v>72</v>
-      </c>
-      <c r="HG176" t="n">
-        <v>18</v>
-      </c>
-      <c r="HH176" t="n">
-        <v>10</v>
-      </c>
-      <c r="HI176" t="n">
+      <c r="HM176" t="n">
+        <v>14</v>
+      </c>
+      <c r="HN176" t="n">
         <v>100</v>
       </c>
-      <c r="HJ176" t="n">
-        <v>8</v>
-      </c>
-      <c r="HK176" t="n">
-        <v>60</v>
-      </c>
-      <c r="HL176" t="n">
-        <v>30</v>
-      </c>
-      <c r="HM176" t="n">
-        <v>10</v>
-      </c>
-      <c r="HN176" t="n">
-        <v>90</v>
-      </c>
       <c r="HO176" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="HP176" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="HQ176" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="HR176" t="n">
         <v>10</v>
       </c>
       <c r="HS176" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="HT176" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="HU176" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="HV176" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="HW176" t="n">
         <v>0</v>
@@ -53458,70 +53528,60 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SAMUEL KIMENYI</t>
+          <t>Southern Mauritania Afforestation - Date Palm Tree</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>SAMUEL KIMENYI</t>
+          <t>El Hadji Beye</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>9720562.16, 753393.14</t>
-        </is>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Mountaine Forest</t>
+          <t>Arid or Semi-Arid Zones</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>Mauritania</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Kigali</t>
+          <t>Kaedi</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Seed Dispersal</t>
+          <t>Full Seedling Plantation (NTFP)</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>seed_dispersal</t>
+          <t>seedling_planting_ntfp</t>
         </is>
       </c>
       <c r="J177" t="n">
-        <v>321</v>
+        <v>8775</v>
       </c>
       <c r="K177" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="L177" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="M177" t="n">
-        <v>9</v>
-      </c>
-      <c r="N177" t="n">
-        <v>2</v>
-      </c>
-      <c r="O177" t="n">
-        <v>20</v>
-      </c>
-      <c r="P177" t="n">
-        <v>70</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
+      <c r="P177" t="inlineStr"/>
       <c r="Q177" t="inlineStr"/>
       <c r="R177" t="inlineStr"/>
       <c r="S177" t="inlineStr"/>
@@ -53549,15 +53609,33 @@
       <c r="AO177" t="inlineStr"/>
       <c r="AP177" t="inlineStr"/>
       <c r="AQ177" t="inlineStr"/>
-      <c r="AR177" t="inlineStr"/>
-      <c r="AS177" t="inlineStr"/>
-      <c r="AT177" t="inlineStr"/>
-      <c r="AU177" t="inlineStr"/>
-      <c r="AV177" t="inlineStr"/>
-      <c r="AW177" t="inlineStr"/>
-      <c r="AX177" t="inlineStr"/>
-      <c r="AY177" t="inlineStr"/>
-      <c r="AZ177" t="inlineStr"/>
+      <c r="AR177" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS177" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT177" t="n">
+        <v>370</v>
+      </c>
+      <c r="AU177" t="n">
+        <v>7</v>
+      </c>
+      <c r="AV177" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW177" t="n">
+        <v>610</v>
+      </c>
+      <c r="AX177" t="n">
+        <v>10</v>
+      </c>
+      <c r="AY177" t="n">
+        <v>20</v>
+      </c>
+      <c r="AZ177" t="n">
+        <v>820</v>
+      </c>
       <c r="BA177" t="inlineStr"/>
       <c r="BB177" t="inlineStr"/>
       <c r="BC177" t="inlineStr"/>
@@ -53579,12 +53657,24 @@
       <c r="BS177" t="inlineStr"/>
       <c r="BT177" t="inlineStr"/>
       <c r="BU177" t="inlineStr"/>
-      <c r="BV177" t="inlineStr"/>
-      <c r="BW177" t="inlineStr"/>
-      <c r="BX177" t="inlineStr"/>
-      <c r="BY177" t="inlineStr"/>
-      <c r="BZ177" t="inlineStr"/>
-      <c r="CA177" t="inlineStr"/>
+      <c r="BV177" t="n">
+        <v>6</v>
+      </c>
+      <c r="BW177" t="n">
+        <v>9</v>
+      </c>
+      <c r="BX177" t="n">
+        <v>395</v>
+      </c>
+      <c r="BY177" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ177" t="n">
+        <v>20</v>
+      </c>
+      <c r="CA177" t="n">
+        <v>550</v>
+      </c>
       <c r="CB177" t="inlineStr"/>
       <c r="CC177" t="inlineStr"/>
       <c r="CD177" t="inlineStr"/>
@@ -53616,7 +53706,7 @@
         <v>20</v>
       </c>
       <c r="DB177" t="n">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="DC177" t="inlineStr"/>
       <c r="DD177" t="inlineStr"/>
@@ -53652,7 +53742,7 @@
         <v>20</v>
       </c>
       <c r="EF177" t="n">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="EG177" t="inlineStr"/>
       <c r="EH177" t="inlineStr"/>
@@ -53682,16 +53772,22 @@
       <c r="FF177" t="inlineStr"/>
       <c r="FG177" t="inlineStr"/>
       <c r="FH177" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="FI177" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="FJ177" t="n">
-        <v>6</v>
-      </c>
-      <c r="FK177" t="inlineStr"/>
-      <c r="FL177" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="FK177" t="inlineStr">
+        <is>
+          <t>Date palm Tree (Phoenix dactylifera)</t>
+        </is>
+      </c>
+      <c r="FL177" t="n">
+        <v>2.89</v>
+      </c>
       <c r="FM177" t="inlineStr"/>
       <c r="FN177" t="inlineStr"/>
       <c r="FO177" t="inlineStr"/>
@@ -53707,15 +53803,33 @@
       <c r="FY177" t="inlineStr"/>
       <c r="FZ177" t="inlineStr"/>
       <c r="GA177" t="inlineStr"/>
-      <c r="GB177" t="inlineStr"/>
-      <c r="GC177" t="inlineStr"/>
-      <c r="GD177" t="inlineStr"/>
-      <c r="GE177" t="inlineStr"/>
-      <c r="GF177" t="inlineStr"/>
-      <c r="GG177" t="inlineStr"/>
-      <c r="GH177" t="inlineStr"/>
-      <c r="GI177" t="inlineStr"/>
-      <c r="GJ177" t="inlineStr"/>
+      <c r="GB177" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC177" t="n">
+        <v>6</v>
+      </c>
+      <c r="GD177" t="n">
+        <v>0</v>
+      </c>
+      <c r="GE177" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF177" t="n">
+        <v>9</v>
+      </c>
+      <c r="GG177" t="n">
+        <v>13845</v>
+      </c>
+      <c r="GH177" t="n">
+        <v>10</v>
+      </c>
+      <c r="GI177" t="n">
+        <v>20</v>
+      </c>
+      <c r="GJ177" t="n">
+        <v>23779</v>
+      </c>
       <c r="GK177" t="inlineStr"/>
       <c r="GL177" t="inlineStr"/>
       <c r="GM177" t="inlineStr"/>
@@ -53723,100 +53837,100 @@
       <c r="GO177" t="inlineStr"/>
       <c r="GP177" t="inlineStr"/>
       <c r="GQ177" t="n">
-        <v>3447.15</v>
+        <v>252.98</v>
       </c>
       <c r="GR177" t="n">
-        <v>975.001256306883</v>
+        <v>31.99972009877586</v>
       </c>
       <c r="GS177" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="GT177" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="GU177" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="GV177" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="GW177" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="GX177" t="n">
-        <v>4027.02</v>
+        <v>1000</v>
       </c>
       <c r="GY177" t="n">
-        <v>930.0004324128028</v>
+        <v>400</v>
       </c>
       <c r="GZ177" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="HA177" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="HB177" t="n">
+        <v>32</v>
+      </c>
+      <c r="HC177" t="n">
+        <v>9</v>
+      </c>
+      <c r="HD177" t="n">
+        <v>140</v>
+      </c>
+      <c r="HE177" t="n">
+        <v>10</v>
+      </c>
+      <c r="HF177" t="n">
+        <v>43</v>
+      </c>
+      <c r="HG177" t="n">
+        <v>43</v>
+      </c>
+      <c r="HH177" t="n">
+        <v>14</v>
+      </c>
+      <c r="HI177" t="n">
+        <v>116</v>
+      </c>
+      <c r="HJ177" t="n">
+        <v>15</v>
+      </c>
+      <c r="HK177" t="n">
+        <v>51</v>
+      </c>
+      <c r="HL177" t="n">
         <v>35</v>
       </c>
-      <c r="HC177" t="n">
-        <v>5</v>
-      </c>
-      <c r="HD177" t="n">
-        <v>150</v>
-      </c>
-      <c r="HE177" t="n">
-        <v>20</v>
-      </c>
-      <c r="HF177" t="n">
-        <v>72</v>
-      </c>
-      <c r="HG177" t="n">
-        <v>18</v>
-      </c>
-      <c r="HH177" t="n">
-        <v>10</v>
-      </c>
-      <c r="HI177" t="n">
+      <c r="HM177" t="n">
+        <v>14</v>
+      </c>
+      <c r="HN177" t="n">
         <v>100</v>
       </c>
-      <c r="HJ177" t="n">
-        <v>8</v>
-      </c>
-      <c r="HK177" t="n">
-        <v>60</v>
-      </c>
-      <c r="HL177" t="n">
-        <v>30</v>
-      </c>
-      <c r="HM177" t="n">
-        <v>10</v>
-      </c>
-      <c r="HN177" t="n">
-        <v>90</v>
-      </c>
       <c r="HO177" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="HP177" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="HQ177" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="HR177" t="n">
         <v>10</v>
       </c>
       <c r="HS177" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="HT177" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="HU177" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="HV177" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="HW177" t="n">
         <v>0</v>
@@ -53860,29 +53974,35 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Seed Dispersal (NTFP)</t>
+          <t>ANR/50% Enrichment</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>seed_dispersal_ntfp</t>
+          <t>anr_30</t>
         </is>
       </c>
       <c r="J178" t="n">
-        <v>430</v>
+        <v>651</v>
       </c>
       <c r="K178" t="n">
         <v>57</v>
       </c>
       <c r="L178" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M178" t="n">
-        <v>9</v>
-      </c>
-      <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr"/>
-      <c r="P178" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="N178" t="n">
+        <v>2</v>
+      </c>
+      <c r="O178" t="n">
+        <v>20</v>
+      </c>
+      <c r="P178" t="n">
+        <v>100</v>
+      </c>
       <c r="Q178" t="inlineStr"/>
       <c r="R178" t="inlineStr"/>
       <c r="S178" t="inlineStr"/>
@@ -53910,15 +54030,9 @@
       <c r="AO178" t="inlineStr"/>
       <c r="AP178" t="inlineStr"/>
       <c r="AQ178" t="inlineStr"/>
-      <c r="AR178" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS178" t="n">
-        <v>20</v>
-      </c>
-      <c r="AT178" t="n">
-        <v>165</v>
-      </c>
+      <c r="AR178" t="inlineStr"/>
+      <c r="AS178" t="inlineStr"/>
+      <c r="AT178" t="inlineStr"/>
       <c r="AU178" t="inlineStr"/>
       <c r="AV178" t="inlineStr"/>
       <c r="AW178" t="inlineStr"/>
@@ -53946,15 +54060,9 @@
       <c r="BS178" t="inlineStr"/>
       <c r="BT178" t="inlineStr"/>
       <c r="BU178" t="inlineStr"/>
-      <c r="BV178" t="n">
-        <v>5</v>
-      </c>
-      <c r="BW178" t="n">
-        <v>20</v>
-      </c>
-      <c r="BX178" t="n">
-        <v>110</v>
-      </c>
+      <c r="BV178" t="inlineStr"/>
+      <c r="BW178" t="inlineStr"/>
+      <c r="BX178" t="inlineStr"/>
       <c r="BY178" t="inlineStr"/>
       <c r="BZ178" t="inlineStr"/>
       <c r="CA178" t="inlineStr"/>
@@ -53989,7 +54097,7 @@
         <v>20</v>
       </c>
       <c r="DB178" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="DC178" t="inlineStr"/>
       <c r="DD178" t="inlineStr"/>
@@ -54055,58 +54163,28 @@
       <c r="FF178" t="inlineStr"/>
       <c r="FG178" t="inlineStr"/>
       <c r="FH178" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="FI178" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="FJ178" t="n">
-        <v>13</v>
-      </c>
-      <c r="FK178" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Yushania alpina</t>
-        </is>
-      </c>
-      <c r="FL178" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="FM178" t="n">
-        <v>5</v>
-      </c>
-      <c r="FN178" t="n">
-        <v>9</v>
-      </c>
-      <c r="FO178" t="n">
-        <v>1200</v>
-      </c>
-      <c r="FP178" t="n">
-        <v>10</v>
-      </c>
-      <c r="FQ178" t="n">
-        <v>14</v>
-      </c>
-      <c r="FR178" t="n">
-        <v>3600</v>
-      </c>
-      <c r="FS178" t="n">
-        <v>15</v>
-      </c>
-      <c r="FT178" t="n">
-        <v>19</v>
-      </c>
-      <c r="FU178" t="n">
-        <v>5600</v>
-      </c>
-      <c r="FV178" t="n">
-        <v>19</v>
-      </c>
-      <c r="FW178" t="n">
-        <v>20</v>
-      </c>
-      <c r="FX178" t="n">
-        <v>6400</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="FK178" t="inlineStr"/>
+      <c r="FL178" t="inlineStr"/>
+      <c r="FM178" t="inlineStr"/>
+      <c r="FN178" t="inlineStr"/>
+      <c r="FO178" t="inlineStr"/>
+      <c r="FP178" t="inlineStr"/>
+      <c r="FQ178" t="inlineStr"/>
+      <c r="FR178" t="inlineStr"/>
+      <c r="FS178" t="inlineStr"/>
+      <c r="FT178" t="inlineStr"/>
+      <c r="FU178" t="inlineStr"/>
+      <c r="FV178" t="inlineStr"/>
+      <c r="FW178" t="inlineStr"/>
+      <c r="FX178" t="inlineStr"/>
       <c r="FY178" t="inlineStr"/>
       <c r="FZ178" t="inlineStr"/>
       <c r="GA178" t="inlineStr"/>
@@ -54263,35 +54341,29 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Full Seedling Plantation</t>
+          <t>ANR/50% Enrichment (NTFP)</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>seedling_planting</t>
+          <t>anr_30_ntfp</t>
         </is>
       </c>
       <c r="J179" t="n">
-        <v>1250</v>
+        <v>785</v>
       </c>
       <c r="K179" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L179" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M179" t="n">
-        <v>10</v>
-      </c>
-      <c r="N179" t="n">
-        <v>2</v>
-      </c>
-      <c r="O179" t="n">
-        <v>20</v>
-      </c>
-      <c r="P179" t="n">
-        <v>245</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
+      <c r="P179" t="inlineStr"/>
       <c r="Q179" t="inlineStr"/>
       <c r="R179" t="inlineStr"/>
       <c r="S179" t="inlineStr"/>
@@ -54319,9 +54391,15 @@
       <c r="AO179" t="inlineStr"/>
       <c r="AP179" t="inlineStr"/>
       <c r="AQ179" t="inlineStr"/>
-      <c r="AR179" t="inlineStr"/>
-      <c r="AS179" t="inlineStr"/>
-      <c r="AT179" t="inlineStr"/>
+      <c r="AR179" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS179" t="n">
+        <v>20</v>
+      </c>
+      <c r="AT179" t="n">
+        <v>163</v>
+      </c>
       <c r="AU179" t="inlineStr"/>
       <c r="AV179" t="inlineStr"/>
       <c r="AW179" t="inlineStr"/>
@@ -54349,9 +54427,15 @@
       <c r="BS179" t="inlineStr"/>
       <c r="BT179" t="inlineStr"/>
       <c r="BU179" t="inlineStr"/>
-      <c r="BV179" t="inlineStr"/>
-      <c r="BW179" t="inlineStr"/>
-      <c r="BX179" t="inlineStr"/>
+      <c r="BV179" t="n">
+        <v>5</v>
+      </c>
+      <c r="BW179" t="n">
+        <v>20</v>
+      </c>
+      <c r="BX179" t="n">
+        <v>150</v>
+      </c>
       <c r="BY179" t="inlineStr"/>
       <c r="BZ179" t="inlineStr"/>
       <c r="CA179" t="inlineStr"/>
@@ -54386,7 +54470,7 @@
         <v>20</v>
       </c>
       <c r="DB179" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="DC179" t="inlineStr"/>
       <c r="DD179" t="inlineStr"/>
@@ -54422,7 +54506,7 @@
         <v>20</v>
       </c>
       <c r="EF179" t="n">
-        <v>250</v>
+        <v>390</v>
       </c>
       <c r="EG179" t="inlineStr"/>
       <c r="EH179" t="inlineStr"/>
@@ -54452,28 +54536,58 @@
       <c r="FF179" t="inlineStr"/>
       <c r="FG179" t="inlineStr"/>
       <c r="FH179" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="FI179" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="FJ179" t="n">
-        <v>7</v>
-      </c>
-      <c r="FK179" t="inlineStr"/>
-      <c r="FL179" t="inlineStr"/>
-      <c r="FM179" t="inlineStr"/>
-      <c r="FN179" t="inlineStr"/>
-      <c r="FO179" t="inlineStr"/>
-      <c r="FP179" t="inlineStr"/>
-      <c r="FQ179" t="inlineStr"/>
-      <c r="FR179" t="inlineStr"/>
-      <c r="FS179" t="inlineStr"/>
-      <c r="FT179" t="inlineStr"/>
-      <c r="FU179" t="inlineStr"/>
-      <c r="FV179" t="inlineStr"/>
-      <c r="FW179" t="inlineStr"/>
-      <c r="FX179" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="FK179" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Yushania alpina</t>
+        </is>
+      </c>
+      <c r="FL179" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="FM179" t="n">
+        <v>5</v>
+      </c>
+      <c r="FN179" t="n">
+        <v>9</v>
+      </c>
+      <c r="FO179" t="n">
+        <v>4100</v>
+      </c>
+      <c r="FP179" t="n">
+        <v>10</v>
+      </c>
+      <c r="FQ179" t="n">
+        <v>14</v>
+      </c>
+      <c r="FR179" t="n">
+        <v>8400</v>
+      </c>
+      <c r="FS179" t="n">
+        <v>15</v>
+      </c>
+      <c r="FT179" t="n">
+        <v>19</v>
+      </c>
+      <c r="FU179" t="n">
+        <v>11300</v>
+      </c>
+      <c r="FV179" t="n">
+        <v>20</v>
+      </c>
+      <c r="FW179" t="n">
+        <v>20</v>
+      </c>
+      <c r="FX179" t="n">
+        <v>13500</v>
+      </c>
       <c r="FY179" t="inlineStr"/>
       <c r="FZ179" t="inlineStr"/>
       <c r="GA179" t="inlineStr"/>
@@ -54630,29 +54744,35 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Full Seedling Plantation (NTFP)</t>
+          <t>Seed Dispersal</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>seedling_planting_ntfp</t>
+          <t>seed_dispersal</t>
         </is>
       </c>
       <c r="J180" t="n">
-        <v>1530</v>
+        <v>321</v>
       </c>
       <c r="K180" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="L180" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="M180" t="n">
-        <v>8</v>
-      </c>
-      <c r="N180" t="inlineStr"/>
-      <c r="O180" t="inlineStr"/>
-      <c r="P180" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="N180" t="n">
+        <v>2</v>
+      </c>
+      <c r="O180" t="n">
+        <v>20</v>
+      </c>
+      <c r="P180" t="n">
+        <v>70</v>
+      </c>
       <c r="Q180" t="inlineStr"/>
       <c r="R180" t="inlineStr"/>
       <c r="S180" t="inlineStr"/>
@@ -54680,15 +54800,9 @@
       <c r="AO180" t="inlineStr"/>
       <c r="AP180" t="inlineStr"/>
       <c r="AQ180" t="inlineStr"/>
-      <c r="AR180" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS180" t="n">
-        <v>20</v>
-      </c>
-      <c r="AT180" t="n">
-        <v>260</v>
-      </c>
+      <c r="AR180" t="inlineStr"/>
+      <c r="AS180" t="inlineStr"/>
+      <c r="AT180" t="inlineStr"/>
       <c r="AU180" t="inlineStr"/>
       <c r="AV180" t="inlineStr"/>
       <c r="AW180" t="inlineStr"/>
@@ -54716,15 +54830,9 @@
       <c r="BS180" t="inlineStr"/>
       <c r="BT180" t="inlineStr"/>
       <c r="BU180" t="inlineStr"/>
-      <c r="BV180" t="n">
-        <v>5</v>
-      </c>
-      <c r="BW180" t="n">
-        <v>20</v>
-      </c>
-      <c r="BX180" t="n">
-        <v>140</v>
-      </c>
+      <c r="BV180" t="inlineStr"/>
+      <c r="BW180" t="inlineStr"/>
+      <c r="BX180" t="inlineStr"/>
       <c r="BY180" t="inlineStr"/>
       <c r="BZ180" t="inlineStr"/>
       <c r="CA180" t="inlineStr"/>
@@ -54759,7 +54867,7 @@
         <v>20</v>
       </c>
       <c r="DB180" t="n">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="DC180" t="inlineStr"/>
       <c r="DD180" t="inlineStr"/>
@@ -54795,7 +54903,7 @@
         <v>20</v>
       </c>
       <c r="EF180" t="n">
-        <v>330</v>
+        <v>190</v>
       </c>
       <c r="EG180" t="inlineStr"/>
       <c r="EH180" t="inlineStr"/>
@@ -54825,58 +54933,28 @@
       <c r="FF180" t="inlineStr"/>
       <c r="FG180" t="inlineStr"/>
       <c r="FH180" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="FI180" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="FJ180" t="n">
-        <v>13</v>
-      </c>
-      <c r="FK180" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Yushania alpina</t>
-        </is>
-      </c>
-      <c r="FL180" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="FM180" t="n">
-        <v>5</v>
-      </c>
-      <c r="FN180" t="n">
-        <v>9</v>
-      </c>
-      <c r="FO180" t="n">
-        <v>9500</v>
-      </c>
-      <c r="FP180" t="n">
-        <v>10</v>
-      </c>
-      <c r="FQ180" t="n">
-        <v>14</v>
-      </c>
-      <c r="FR180" t="n">
-        <v>18800</v>
-      </c>
-      <c r="FS180" t="n">
-        <v>15</v>
-      </c>
-      <c r="FT180" t="n">
-        <v>19</v>
-      </c>
-      <c r="FU180" t="n">
-        <v>26300</v>
-      </c>
-      <c r="FV180" t="n">
-        <v>19</v>
-      </c>
-      <c r="FW180" t="n">
-        <v>20</v>
-      </c>
-      <c r="FX180" t="n">
-        <v>29800</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="FK180" t="inlineStr"/>
+      <c r="FL180" t="inlineStr"/>
+      <c r="FM180" t="inlineStr"/>
+      <c r="FN180" t="inlineStr"/>
+      <c r="FO180" t="inlineStr"/>
+      <c r="FP180" t="inlineStr"/>
+      <c r="FQ180" t="inlineStr"/>
+      <c r="FR180" t="inlineStr"/>
+      <c r="FS180" t="inlineStr"/>
+      <c r="FT180" t="inlineStr"/>
+      <c r="FU180" t="inlineStr"/>
+      <c r="FV180" t="inlineStr"/>
+      <c r="FW180" t="inlineStr"/>
+      <c r="FX180" t="inlineStr"/>
       <c r="FY180" t="inlineStr"/>
       <c r="FZ180" t="inlineStr"/>
       <c r="GA180" t="inlineStr"/>
@@ -54998,56 +55076,60 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Rede de Sementes RNAPFNM</t>
+          <t>SAMUEL KIMENYI</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Pedro Pereira Santos</t>
+          <t>SAMUEL KIMENYI</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2023-06-06</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr"/>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>9720562.16, 753393.14</t>
+        </is>
+      </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Savanna or Dry Forest</t>
+          <t>Mountaine Forest</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Rwanda</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Alto Paraiso</t>
+          <t>Kigali</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>ANR/50% Enrichment (NTFP)</t>
+          <t>Seed Dispersal (NTFP)</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>anr_30_ntfp</t>
+          <t>seed_dispersal_ntfp</t>
         </is>
       </c>
       <c r="J181" t="n">
-        <v>822.91</v>
+        <v>430</v>
       </c>
       <c r="K181" t="n">
-        <v>24.1</v>
+        <v>57</v>
       </c>
       <c r="L181" t="n">
-        <v>75.90000000000001</v>
+        <v>34</v>
       </c>
       <c r="M181" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N181" t="inlineStr"/>
       <c r="O181" t="inlineStr"/>
@@ -55086,7 +55168,7 @@
         <v>20</v>
       </c>
       <c r="AT181" t="n">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="AU181" t="inlineStr"/>
       <c r="AV181" t="inlineStr"/>
@@ -55115,9 +55197,15 @@
       <c r="BS181" t="inlineStr"/>
       <c r="BT181" t="inlineStr"/>
       <c r="BU181" t="inlineStr"/>
-      <c r="BV181" t="inlineStr"/>
-      <c r="BW181" t="inlineStr"/>
-      <c r="BX181" t="inlineStr"/>
+      <c r="BV181" t="n">
+        <v>5</v>
+      </c>
+      <c r="BW181" t="n">
+        <v>20</v>
+      </c>
+      <c r="BX181" t="n">
+        <v>110</v>
+      </c>
       <c r="BY181" t="inlineStr"/>
       <c r="BZ181" t="inlineStr"/>
       <c r="CA181" t="inlineStr"/>
@@ -55145,9 +55233,15 @@
       <c r="CW181" t="inlineStr"/>
       <c r="CX181" t="inlineStr"/>
       <c r="CY181" t="inlineStr"/>
-      <c r="CZ181" t="inlineStr"/>
-      <c r="DA181" t="inlineStr"/>
-      <c r="DB181" t="inlineStr"/>
+      <c r="CZ181" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA181" t="n">
+        <v>20</v>
+      </c>
+      <c r="DB181" t="n">
+        <v>220</v>
+      </c>
       <c r="DC181" t="inlineStr"/>
       <c r="DD181" t="inlineStr"/>
       <c r="DE181" t="inlineStr"/>
@@ -55179,10 +55273,10 @@
         <v>2</v>
       </c>
       <c r="EE181" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="EF181" t="n">
-        <v>128.09</v>
+        <v>220</v>
       </c>
       <c r="EG181" t="inlineStr"/>
       <c r="EH181" t="inlineStr"/>
@@ -55212,40 +55306,58 @@
       <c r="FF181" t="inlineStr"/>
       <c r="FG181" t="inlineStr"/>
       <c r="FH181" t="n">
-        <v>80.2</v>
+        <v>67</v>
       </c>
       <c r="FI181" t="n">
-        <v>19.8</v>
+        <v>20</v>
       </c>
       <c r="FJ181" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="FK181" t="inlineStr">
         <is>
-          <t>Pequi (Caryocar brasiliense)</t>
+          <t xml:space="preserve"> Yushania alpina</t>
         </is>
       </c>
       <c r="FL181" t="n">
-        <v>0.13</v>
+        <v>0.5</v>
       </c>
       <c r="FM181" t="n">
+        <v>5</v>
+      </c>
+      <c r="FN181" t="n">
+        <v>9</v>
+      </c>
+      <c r="FO181" t="n">
+        <v>1200</v>
+      </c>
+      <c r="FP181" t="n">
         <v>10</v>
       </c>
-      <c r="FN181" t="n">
+      <c r="FQ181" t="n">
+        <v>14</v>
+      </c>
+      <c r="FR181" t="n">
+        <v>3600</v>
+      </c>
+      <c r="FS181" t="n">
+        <v>15</v>
+      </c>
+      <c r="FT181" t="n">
+        <v>19</v>
+      </c>
+      <c r="FU181" t="n">
+        <v>5600</v>
+      </c>
+      <c r="FV181" t="n">
+        <v>19</v>
+      </c>
+      <c r="FW181" t="n">
         <v>20</v>
       </c>
-      <c r="FO181" t="n">
-        <v>900</v>
-      </c>
-      <c r="FP181" t="inlineStr"/>
-      <c r="FQ181" t="inlineStr"/>
-      <c r="FR181" t="inlineStr"/>
-      <c r="FS181" t="inlineStr"/>
-      <c r="FT181" t="inlineStr"/>
-      <c r="FU181" t="inlineStr"/>
-      <c r="FV181" t="inlineStr"/>
-      <c r="FW181" t="inlineStr"/>
-      <c r="FX181" t="inlineStr"/>
+      <c r="FX181" t="n">
+        <v>6400</v>
+      </c>
       <c r="FY181" t="inlineStr"/>
       <c r="FZ181" t="inlineStr"/>
       <c r="GA181" t="inlineStr"/>
@@ -55265,98 +55377,1237 @@
       <c r="GO181" t="inlineStr"/>
       <c r="GP181" t="inlineStr"/>
       <c r="GQ181" t="n">
+        <v>3447.15</v>
+      </c>
+      <c r="GR181" t="n">
+        <v>975.001256306883</v>
+      </c>
+      <c r="GS181" t="n">
+        <v>5</v>
+      </c>
+      <c r="GT181" t="n">
+        <v>2</v>
+      </c>
+      <c r="GU181" t="n">
+        <v>70</v>
+      </c>
+      <c r="GV181" t="n">
+        <v>12</v>
+      </c>
+      <c r="GW181" t="n">
+        <v>18</v>
+      </c>
+      <c r="GX181" t="n">
+        <v>4027.02</v>
+      </c>
+      <c r="GY181" t="n">
+        <v>930.0004324128028</v>
+      </c>
+      <c r="GZ181" t="n">
+        <v>3</v>
+      </c>
+      <c r="HA181" t="n">
+        <v>60</v>
+      </c>
+      <c r="HB181" t="n">
+        <v>35</v>
+      </c>
+      <c r="HC181" t="n">
+        <v>5</v>
+      </c>
+      <c r="HD181" t="n">
+        <v>150</v>
+      </c>
+      <c r="HE181" t="n">
+        <v>20</v>
+      </c>
+      <c r="HF181" t="n">
+        <v>72</v>
+      </c>
+      <c r="HG181" t="n">
+        <v>18</v>
+      </c>
+      <c r="HH181" t="n">
+        <v>10</v>
+      </c>
+      <c r="HI181" t="n">
+        <v>100</v>
+      </c>
+      <c r="HJ181" t="n">
+        <v>8</v>
+      </c>
+      <c r="HK181" t="n">
+        <v>60</v>
+      </c>
+      <c r="HL181" t="n">
+        <v>30</v>
+      </c>
+      <c r="HM181" t="n">
+        <v>10</v>
+      </c>
+      <c r="HN181" t="n">
+        <v>90</v>
+      </c>
+      <c r="HO181" t="n">
+        <v>10</v>
+      </c>
+      <c r="HP181" t="n">
+        <v>60</v>
+      </c>
+      <c r="HQ181" t="n">
+        <v>40</v>
+      </c>
+      <c r="HR181" t="n">
+        <v>10</v>
+      </c>
+      <c r="HS181" t="n">
+        <v>10</v>
+      </c>
+      <c r="HT181" t="n">
+        <v>180</v>
+      </c>
+      <c r="HU181" t="n">
+        <v>70</v>
+      </c>
+      <c r="HV181" t="n">
+        <v>30</v>
+      </c>
+      <c r="HW181" t="n">
         <v>0</v>
       </c>
-      <c r="GR181" t="inlineStr"/>
-      <c r="GS181" t="n">
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>SAMUEL KIMENYI</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>SAMUEL KIMENYI</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>9720562.16, 753393.14</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Mountaine Forest</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Kigali</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Full Seedling Plantation</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>seedling_planting</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>1250</v>
+      </c>
+      <c r="K182" t="n">
+        <v>50</v>
+      </c>
+      <c r="L182" t="n">
+        <v>40</v>
+      </c>
+      <c r="M182" t="n">
+        <v>10</v>
+      </c>
+      <c r="N182" t="n">
+        <v>2</v>
+      </c>
+      <c r="O182" t="n">
+        <v>20</v>
+      </c>
+      <c r="P182" t="n">
+        <v>245</v>
+      </c>
+      <c r="Q182" t="inlineStr"/>
+      <c r="R182" t="inlineStr"/>
+      <c r="S182" t="inlineStr"/>
+      <c r="T182" t="inlineStr"/>
+      <c r="U182" t="inlineStr"/>
+      <c r="V182" t="inlineStr"/>
+      <c r="W182" t="inlineStr"/>
+      <c r="X182" t="inlineStr"/>
+      <c r="Y182" t="inlineStr"/>
+      <c r="Z182" t="inlineStr"/>
+      <c r="AA182" t="inlineStr"/>
+      <c r="AB182" t="inlineStr"/>
+      <c r="AC182" t="inlineStr"/>
+      <c r="AD182" t="inlineStr"/>
+      <c r="AE182" t="inlineStr"/>
+      <c r="AF182" t="inlineStr"/>
+      <c r="AG182" t="inlineStr"/>
+      <c r="AH182" t="inlineStr"/>
+      <c r="AI182" t="inlineStr"/>
+      <c r="AJ182" t="inlineStr"/>
+      <c r="AK182" t="inlineStr"/>
+      <c r="AL182" t="inlineStr"/>
+      <c r="AM182" t="inlineStr"/>
+      <c r="AN182" t="inlineStr"/>
+      <c r="AO182" t="inlineStr"/>
+      <c r="AP182" t="inlineStr"/>
+      <c r="AQ182" t="inlineStr"/>
+      <c r="AR182" t="inlineStr"/>
+      <c r="AS182" t="inlineStr"/>
+      <c r="AT182" t="inlineStr"/>
+      <c r="AU182" t="inlineStr"/>
+      <c r="AV182" t="inlineStr"/>
+      <c r="AW182" t="inlineStr"/>
+      <c r="AX182" t="inlineStr"/>
+      <c r="AY182" t="inlineStr"/>
+      <c r="AZ182" t="inlineStr"/>
+      <c r="BA182" t="inlineStr"/>
+      <c r="BB182" t="inlineStr"/>
+      <c r="BC182" t="inlineStr"/>
+      <c r="BD182" t="inlineStr"/>
+      <c r="BE182" t="inlineStr"/>
+      <c r="BF182" t="inlineStr"/>
+      <c r="BG182" t="inlineStr"/>
+      <c r="BH182" t="inlineStr"/>
+      <c r="BI182" t="inlineStr"/>
+      <c r="BJ182" t="inlineStr"/>
+      <c r="BK182" t="inlineStr"/>
+      <c r="BL182" t="inlineStr"/>
+      <c r="BM182" t="inlineStr"/>
+      <c r="BN182" t="inlineStr"/>
+      <c r="BO182" t="inlineStr"/>
+      <c r="BP182" t="inlineStr"/>
+      <c r="BQ182" t="inlineStr"/>
+      <c r="BR182" t="inlineStr"/>
+      <c r="BS182" t="inlineStr"/>
+      <c r="BT182" t="inlineStr"/>
+      <c r="BU182" t="inlineStr"/>
+      <c r="BV182" t="inlineStr"/>
+      <c r="BW182" t="inlineStr"/>
+      <c r="BX182" t="inlineStr"/>
+      <c r="BY182" t="inlineStr"/>
+      <c r="BZ182" t="inlineStr"/>
+      <c r="CA182" t="inlineStr"/>
+      <c r="CB182" t="inlineStr"/>
+      <c r="CC182" t="inlineStr"/>
+      <c r="CD182" t="inlineStr"/>
+      <c r="CE182" t="inlineStr"/>
+      <c r="CF182" t="inlineStr"/>
+      <c r="CG182" t="inlineStr"/>
+      <c r="CH182" t="inlineStr"/>
+      <c r="CI182" t="inlineStr"/>
+      <c r="CJ182" t="inlineStr"/>
+      <c r="CK182" t="inlineStr"/>
+      <c r="CL182" t="inlineStr"/>
+      <c r="CM182" t="inlineStr"/>
+      <c r="CN182" t="inlineStr"/>
+      <c r="CO182" t="inlineStr"/>
+      <c r="CP182" t="inlineStr"/>
+      <c r="CQ182" t="inlineStr"/>
+      <c r="CR182" t="inlineStr"/>
+      <c r="CS182" t="inlineStr"/>
+      <c r="CT182" t="inlineStr"/>
+      <c r="CU182" t="inlineStr"/>
+      <c r="CV182" t="inlineStr"/>
+      <c r="CW182" t="inlineStr"/>
+      <c r="CX182" t="inlineStr"/>
+      <c r="CY182" t="inlineStr"/>
+      <c r="CZ182" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA182" t="n">
+        <v>20</v>
+      </c>
+      <c r="DB182" t="n">
+        <v>300</v>
+      </c>
+      <c r="DC182" t="inlineStr"/>
+      <c r="DD182" t="inlineStr"/>
+      <c r="DE182" t="inlineStr"/>
+      <c r="DF182" t="inlineStr"/>
+      <c r="DG182" t="inlineStr"/>
+      <c r="DH182" t="inlineStr"/>
+      <c r="DI182" t="inlineStr"/>
+      <c r="DJ182" t="inlineStr"/>
+      <c r="DK182" t="inlineStr"/>
+      <c r="DL182" t="inlineStr"/>
+      <c r="DM182" t="inlineStr"/>
+      <c r="DN182" t="inlineStr"/>
+      <c r="DO182" t="inlineStr"/>
+      <c r="DP182" t="inlineStr"/>
+      <c r="DQ182" t="inlineStr"/>
+      <c r="DR182" t="inlineStr"/>
+      <c r="DS182" t="inlineStr"/>
+      <c r="DT182" t="inlineStr"/>
+      <c r="DU182" t="inlineStr"/>
+      <c r="DV182" t="inlineStr"/>
+      <c r="DW182" t="inlineStr"/>
+      <c r="DX182" t="inlineStr"/>
+      <c r="DY182" t="inlineStr"/>
+      <c r="DZ182" t="inlineStr"/>
+      <c r="EA182" t="inlineStr"/>
+      <c r="EB182" t="inlineStr"/>
+      <c r="EC182" t="inlineStr"/>
+      <c r="ED182" t="n">
+        <v>2</v>
+      </c>
+      <c r="EE182" t="n">
+        <v>20</v>
+      </c>
+      <c r="EF182" t="n">
+        <v>250</v>
+      </c>
+      <c r="EG182" t="inlineStr"/>
+      <c r="EH182" t="inlineStr"/>
+      <c r="EI182" t="inlineStr"/>
+      <c r="EJ182" t="inlineStr"/>
+      <c r="EK182" t="inlineStr"/>
+      <c r="EL182" t="inlineStr"/>
+      <c r="EM182" t="inlineStr"/>
+      <c r="EN182" t="inlineStr"/>
+      <c r="EO182" t="inlineStr"/>
+      <c r="EP182" t="inlineStr"/>
+      <c r="EQ182" t="inlineStr"/>
+      <c r="ER182" t="inlineStr"/>
+      <c r="ES182" t="inlineStr"/>
+      <c r="ET182" t="inlineStr"/>
+      <c r="EU182" t="inlineStr"/>
+      <c r="EV182" t="inlineStr"/>
+      <c r="EW182" t="inlineStr"/>
+      <c r="EX182" t="inlineStr"/>
+      <c r="EY182" t="inlineStr"/>
+      <c r="EZ182" t="inlineStr"/>
+      <c r="FA182" t="inlineStr"/>
+      <c r="FB182" t="inlineStr"/>
+      <c r="FC182" t="inlineStr"/>
+      <c r="FD182" t="inlineStr"/>
+      <c r="FE182" t="inlineStr"/>
+      <c r="FF182" t="inlineStr"/>
+      <c r="FG182" t="inlineStr"/>
+      <c r="FH182" t="n">
+        <v>70</v>
+      </c>
+      <c r="FI182" t="n">
+        <v>23</v>
+      </c>
+      <c r="FJ182" t="n">
+        <v>7</v>
+      </c>
+      <c r="FK182" t="inlineStr"/>
+      <c r="FL182" t="inlineStr"/>
+      <c r="FM182" t="inlineStr"/>
+      <c r="FN182" t="inlineStr"/>
+      <c r="FO182" t="inlineStr"/>
+      <c r="FP182" t="inlineStr"/>
+      <c r="FQ182" t="inlineStr"/>
+      <c r="FR182" t="inlineStr"/>
+      <c r="FS182" t="inlineStr"/>
+      <c r="FT182" t="inlineStr"/>
+      <c r="FU182" t="inlineStr"/>
+      <c r="FV182" t="inlineStr"/>
+      <c r="FW182" t="inlineStr"/>
+      <c r="FX182" t="inlineStr"/>
+      <c r="FY182" t="inlineStr"/>
+      <c r="FZ182" t="inlineStr"/>
+      <c r="GA182" t="inlineStr"/>
+      <c r="GB182" t="inlineStr"/>
+      <c r="GC182" t="inlineStr"/>
+      <c r="GD182" t="inlineStr"/>
+      <c r="GE182" t="inlineStr"/>
+      <c r="GF182" t="inlineStr"/>
+      <c r="GG182" t="inlineStr"/>
+      <c r="GH182" t="inlineStr"/>
+      <c r="GI182" t="inlineStr"/>
+      <c r="GJ182" t="inlineStr"/>
+      <c r="GK182" t="inlineStr"/>
+      <c r="GL182" t="inlineStr"/>
+      <c r="GM182" t="inlineStr"/>
+      <c r="GN182" t="inlineStr"/>
+      <c r="GO182" t="inlineStr"/>
+      <c r="GP182" t="inlineStr"/>
+      <c r="GQ182" t="n">
+        <v>3447.15</v>
+      </c>
+      <c r="GR182" t="n">
+        <v>975.001256306883</v>
+      </c>
+      <c r="GS182" t="n">
+        <v>5</v>
+      </c>
+      <c r="GT182" t="n">
+        <v>2</v>
+      </c>
+      <c r="GU182" t="n">
+        <v>70</v>
+      </c>
+      <c r="GV182" t="n">
+        <v>12</v>
+      </c>
+      <c r="GW182" t="n">
+        <v>18</v>
+      </c>
+      <c r="GX182" t="n">
+        <v>4027.02</v>
+      </c>
+      <c r="GY182" t="n">
+        <v>930.0004324128028</v>
+      </c>
+      <c r="GZ182" t="n">
+        <v>3</v>
+      </c>
+      <c r="HA182" t="n">
+        <v>60</v>
+      </c>
+      <c r="HB182" t="n">
+        <v>35</v>
+      </c>
+      <c r="HC182" t="n">
+        <v>5</v>
+      </c>
+      <c r="HD182" t="n">
+        <v>150</v>
+      </c>
+      <c r="HE182" t="n">
+        <v>20</v>
+      </c>
+      <c r="HF182" t="n">
+        <v>72</v>
+      </c>
+      <c r="HG182" t="n">
+        <v>18</v>
+      </c>
+      <c r="HH182" t="n">
+        <v>10</v>
+      </c>
+      <c r="HI182" t="n">
+        <v>100</v>
+      </c>
+      <c r="HJ182" t="n">
+        <v>8</v>
+      </c>
+      <c r="HK182" t="n">
+        <v>60</v>
+      </c>
+      <c r="HL182" t="n">
+        <v>30</v>
+      </c>
+      <c r="HM182" t="n">
+        <v>10</v>
+      </c>
+      <c r="HN182" t="n">
+        <v>90</v>
+      </c>
+      <c r="HO182" t="n">
+        <v>10</v>
+      </c>
+      <c r="HP182" t="n">
+        <v>60</v>
+      </c>
+      <c r="HQ182" t="n">
+        <v>40</v>
+      </c>
+      <c r="HR182" t="n">
+        <v>10</v>
+      </c>
+      <c r="HS182" t="n">
+        <v>10</v>
+      </c>
+      <c r="HT182" t="n">
+        <v>180</v>
+      </c>
+      <c r="HU182" t="n">
+        <v>70</v>
+      </c>
+      <c r="HV182" t="n">
+        <v>30</v>
+      </c>
+      <c r="HW182" t="n">
         <v>0</v>
       </c>
-      <c r="GT181" t="n">
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>SAMUEL KIMENYI</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>SAMUEL KIMENYI</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>9720562.16, 753393.14</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Mountaine Forest</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Kigali</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Full Seedling Plantation (NTFP)</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>seedling_planting_ntfp</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>1530</v>
+      </c>
+      <c r="K183" t="n">
+        <v>46</v>
+      </c>
+      <c r="L183" t="n">
+        <v>46</v>
+      </c>
+      <c r="M183" t="n">
+        <v>8</v>
+      </c>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
+      <c r="P183" t="inlineStr"/>
+      <c r="Q183" t="inlineStr"/>
+      <c r="R183" t="inlineStr"/>
+      <c r="S183" t="inlineStr"/>
+      <c r="T183" t="inlineStr"/>
+      <c r="U183" t="inlineStr"/>
+      <c r="V183" t="inlineStr"/>
+      <c r="W183" t="inlineStr"/>
+      <c r="X183" t="inlineStr"/>
+      <c r="Y183" t="inlineStr"/>
+      <c r="Z183" t="inlineStr"/>
+      <c r="AA183" t="inlineStr"/>
+      <c r="AB183" t="inlineStr"/>
+      <c r="AC183" t="inlineStr"/>
+      <c r="AD183" t="inlineStr"/>
+      <c r="AE183" t="inlineStr"/>
+      <c r="AF183" t="inlineStr"/>
+      <c r="AG183" t="inlineStr"/>
+      <c r="AH183" t="inlineStr"/>
+      <c r="AI183" t="inlineStr"/>
+      <c r="AJ183" t="inlineStr"/>
+      <c r="AK183" t="inlineStr"/>
+      <c r="AL183" t="inlineStr"/>
+      <c r="AM183" t="inlineStr"/>
+      <c r="AN183" t="inlineStr"/>
+      <c r="AO183" t="inlineStr"/>
+      <c r="AP183" t="inlineStr"/>
+      <c r="AQ183" t="inlineStr"/>
+      <c r="AR183" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS183" t="n">
+        <v>20</v>
+      </c>
+      <c r="AT183" t="n">
+        <v>260</v>
+      </c>
+      <c r="AU183" t="inlineStr"/>
+      <c r="AV183" t="inlineStr"/>
+      <c r="AW183" t="inlineStr"/>
+      <c r="AX183" t="inlineStr"/>
+      <c r="AY183" t="inlineStr"/>
+      <c r="AZ183" t="inlineStr"/>
+      <c r="BA183" t="inlineStr"/>
+      <c r="BB183" t="inlineStr"/>
+      <c r="BC183" t="inlineStr"/>
+      <c r="BD183" t="inlineStr"/>
+      <c r="BE183" t="inlineStr"/>
+      <c r="BF183" t="inlineStr"/>
+      <c r="BG183" t="inlineStr"/>
+      <c r="BH183" t="inlineStr"/>
+      <c r="BI183" t="inlineStr"/>
+      <c r="BJ183" t="inlineStr"/>
+      <c r="BK183" t="inlineStr"/>
+      <c r="BL183" t="inlineStr"/>
+      <c r="BM183" t="inlineStr"/>
+      <c r="BN183" t="inlineStr"/>
+      <c r="BO183" t="inlineStr"/>
+      <c r="BP183" t="inlineStr"/>
+      <c r="BQ183" t="inlineStr"/>
+      <c r="BR183" t="inlineStr"/>
+      <c r="BS183" t="inlineStr"/>
+      <c r="BT183" t="inlineStr"/>
+      <c r="BU183" t="inlineStr"/>
+      <c r="BV183" t="n">
+        <v>5</v>
+      </c>
+      <c r="BW183" t="n">
+        <v>20</v>
+      </c>
+      <c r="BX183" t="n">
+        <v>140</v>
+      </c>
+      <c r="BY183" t="inlineStr"/>
+      <c r="BZ183" t="inlineStr"/>
+      <c r="CA183" t="inlineStr"/>
+      <c r="CB183" t="inlineStr"/>
+      <c r="CC183" t="inlineStr"/>
+      <c r="CD183" t="inlineStr"/>
+      <c r="CE183" t="inlineStr"/>
+      <c r="CF183" t="inlineStr"/>
+      <c r="CG183" t="inlineStr"/>
+      <c r="CH183" t="inlineStr"/>
+      <c r="CI183" t="inlineStr"/>
+      <c r="CJ183" t="inlineStr"/>
+      <c r="CK183" t="inlineStr"/>
+      <c r="CL183" t="inlineStr"/>
+      <c r="CM183" t="inlineStr"/>
+      <c r="CN183" t="inlineStr"/>
+      <c r="CO183" t="inlineStr"/>
+      <c r="CP183" t="inlineStr"/>
+      <c r="CQ183" t="inlineStr"/>
+      <c r="CR183" t="inlineStr"/>
+      <c r="CS183" t="inlineStr"/>
+      <c r="CT183" t="inlineStr"/>
+      <c r="CU183" t="inlineStr"/>
+      <c r="CV183" t="inlineStr"/>
+      <c r="CW183" t="inlineStr"/>
+      <c r="CX183" t="inlineStr"/>
+      <c r="CY183" t="inlineStr"/>
+      <c r="CZ183" t="n">
+        <v>2</v>
+      </c>
+      <c r="DA183" t="n">
+        <v>20</v>
+      </c>
+      <c r="DB183" t="n">
+        <v>300</v>
+      </c>
+      <c r="DC183" t="inlineStr"/>
+      <c r="DD183" t="inlineStr"/>
+      <c r="DE183" t="inlineStr"/>
+      <c r="DF183" t="inlineStr"/>
+      <c r="DG183" t="inlineStr"/>
+      <c r="DH183" t="inlineStr"/>
+      <c r="DI183" t="inlineStr"/>
+      <c r="DJ183" t="inlineStr"/>
+      <c r="DK183" t="inlineStr"/>
+      <c r="DL183" t="inlineStr"/>
+      <c r="DM183" t="inlineStr"/>
+      <c r="DN183" t="inlineStr"/>
+      <c r="DO183" t="inlineStr"/>
+      <c r="DP183" t="inlineStr"/>
+      <c r="DQ183" t="inlineStr"/>
+      <c r="DR183" t="inlineStr"/>
+      <c r="DS183" t="inlineStr"/>
+      <c r="DT183" t="inlineStr"/>
+      <c r="DU183" t="inlineStr"/>
+      <c r="DV183" t="inlineStr"/>
+      <c r="DW183" t="inlineStr"/>
+      <c r="DX183" t="inlineStr"/>
+      <c r="DY183" t="inlineStr"/>
+      <c r="DZ183" t="inlineStr"/>
+      <c r="EA183" t="inlineStr"/>
+      <c r="EB183" t="inlineStr"/>
+      <c r="EC183" t="inlineStr"/>
+      <c r="ED183" t="n">
+        <v>2</v>
+      </c>
+      <c r="EE183" t="n">
+        <v>20</v>
+      </c>
+      <c r="EF183" t="n">
+        <v>330</v>
+      </c>
+      <c r="EG183" t="inlineStr"/>
+      <c r="EH183" t="inlineStr"/>
+      <c r="EI183" t="inlineStr"/>
+      <c r="EJ183" t="inlineStr"/>
+      <c r="EK183" t="inlineStr"/>
+      <c r="EL183" t="inlineStr"/>
+      <c r="EM183" t="inlineStr"/>
+      <c r="EN183" t="inlineStr"/>
+      <c r="EO183" t="inlineStr"/>
+      <c r="EP183" t="inlineStr"/>
+      <c r="EQ183" t="inlineStr"/>
+      <c r="ER183" t="inlineStr"/>
+      <c r="ES183" t="inlineStr"/>
+      <c r="ET183" t="inlineStr"/>
+      <c r="EU183" t="inlineStr"/>
+      <c r="EV183" t="inlineStr"/>
+      <c r="EW183" t="inlineStr"/>
+      <c r="EX183" t="inlineStr"/>
+      <c r="EY183" t="inlineStr"/>
+      <c r="EZ183" t="inlineStr"/>
+      <c r="FA183" t="inlineStr"/>
+      <c r="FB183" t="inlineStr"/>
+      <c r="FC183" t="inlineStr"/>
+      <c r="FD183" t="inlineStr"/>
+      <c r="FE183" t="inlineStr"/>
+      <c r="FF183" t="inlineStr"/>
+      <c r="FG183" t="inlineStr"/>
+      <c r="FH183" t="n">
+        <v>63</v>
+      </c>
+      <c r="FI183" t="n">
+        <v>24</v>
+      </c>
+      <c r="FJ183" t="n">
+        <v>13</v>
+      </c>
+      <c r="FK183" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Yushania alpina</t>
+        </is>
+      </c>
+      <c r="FL183" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="FM183" t="n">
+        <v>5</v>
+      </c>
+      <c r="FN183" t="n">
+        <v>9</v>
+      </c>
+      <c r="FO183" t="n">
+        <v>9500</v>
+      </c>
+      <c r="FP183" t="n">
+        <v>10</v>
+      </c>
+      <c r="FQ183" t="n">
+        <v>14</v>
+      </c>
+      <c r="FR183" t="n">
+        <v>18800</v>
+      </c>
+      <c r="FS183" t="n">
+        <v>15</v>
+      </c>
+      <c r="FT183" t="n">
+        <v>19</v>
+      </c>
+      <c r="FU183" t="n">
+        <v>26300</v>
+      </c>
+      <c r="FV183" t="n">
+        <v>19</v>
+      </c>
+      <c r="FW183" t="n">
+        <v>20</v>
+      </c>
+      <c r="FX183" t="n">
+        <v>29800</v>
+      </c>
+      <c r="FY183" t="inlineStr"/>
+      <c r="FZ183" t="inlineStr"/>
+      <c r="GA183" t="inlineStr"/>
+      <c r="GB183" t="inlineStr"/>
+      <c r="GC183" t="inlineStr"/>
+      <c r="GD183" t="inlineStr"/>
+      <c r="GE183" t="inlineStr"/>
+      <c r="GF183" t="inlineStr"/>
+      <c r="GG183" t="inlineStr"/>
+      <c r="GH183" t="inlineStr"/>
+      <c r="GI183" t="inlineStr"/>
+      <c r="GJ183" t="inlineStr"/>
+      <c r="GK183" t="inlineStr"/>
+      <c r="GL183" t="inlineStr"/>
+      <c r="GM183" t="inlineStr"/>
+      <c r="GN183" t="inlineStr"/>
+      <c r="GO183" t="inlineStr"/>
+      <c r="GP183" t="inlineStr"/>
+      <c r="GQ183" t="n">
+        <v>3447.15</v>
+      </c>
+      <c r="GR183" t="n">
+        <v>975.001256306883</v>
+      </c>
+      <c r="GS183" t="n">
+        <v>5</v>
+      </c>
+      <c r="GT183" t="n">
+        <v>2</v>
+      </c>
+      <c r="GU183" t="n">
+        <v>70</v>
+      </c>
+      <c r="GV183" t="n">
+        <v>12</v>
+      </c>
+      <c r="GW183" t="n">
+        <v>18</v>
+      </c>
+      <c r="GX183" t="n">
+        <v>4027.02</v>
+      </c>
+      <c r="GY183" t="n">
+        <v>930.0004324128028</v>
+      </c>
+      <c r="GZ183" t="n">
+        <v>3</v>
+      </c>
+      <c r="HA183" t="n">
+        <v>60</v>
+      </c>
+      <c r="HB183" t="n">
+        <v>35</v>
+      </c>
+      <c r="HC183" t="n">
+        <v>5</v>
+      </c>
+      <c r="HD183" t="n">
+        <v>150</v>
+      </c>
+      <c r="HE183" t="n">
+        <v>20</v>
+      </c>
+      <c r="HF183" t="n">
+        <v>72</v>
+      </c>
+      <c r="HG183" t="n">
+        <v>18</v>
+      </c>
+      <c r="HH183" t="n">
+        <v>10</v>
+      </c>
+      <c r="HI183" t="n">
+        <v>100</v>
+      </c>
+      <c r="HJ183" t="n">
+        <v>8</v>
+      </c>
+      <c r="HK183" t="n">
+        <v>60</v>
+      </c>
+      <c r="HL183" t="n">
+        <v>30</v>
+      </c>
+      <c r="HM183" t="n">
+        <v>10</v>
+      </c>
+      <c r="HN183" t="n">
+        <v>90</v>
+      </c>
+      <c r="HO183" t="n">
+        <v>10</v>
+      </c>
+      <c r="HP183" t="n">
+        <v>60</v>
+      </c>
+      <c r="HQ183" t="n">
+        <v>40</v>
+      </c>
+      <c r="HR183" t="n">
+        <v>10</v>
+      </c>
+      <c r="HS183" t="n">
+        <v>10</v>
+      </c>
+      <c r="HT183" t="n">
+        <v>180</v>
+      </c>
+      <c r="HU183" t="n">
+        <v>70</v>
+      </c>
+      <c r="HV183" t="n">
+        <v>30</v>
+      </c>
+      <c r="HW183" t="n">
         <v>0</v>
       </c>
-      <c r="GU181" t="n">
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Rede de Sementes RNAPFNM</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Pedro Pereira Santos</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>2023-06-06</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Savanna or Dry Forest</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Alto Paraiso</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>ANR/50% Enrichment (NTFP)</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>anr_30_ntfp</t>
+        </is>
+      </c>
+      <c r="J184" t="n">
+        <v>822.91</v>
+      </c>
+      <c r="K184" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="L184" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="M184" t="n">
         <v>0</v>
       </c>
-      <c r="GV181" t="n">
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
+      <c r="P184" t="inlineStr"/>
+      <c r="Q184" t="inlineStr"/>
+      <c r="R184" t="inlineStr"/>
+      <c r="S184" t="inlineStr"/>
+      <c r="T184" t="inlineStr"/>
+      <c r="U184" t="inlineStr"/>
+      <c r="V184" t="inlineStr"/>
+      <c r="W184" t="inlineStr"/>
+      <c r="X184" t="inlineStr"/>
+      <c r="Y184" t="inlineStr"/>
+      <c r="Z184" t="inlineStr"/>
+      <c r="AA184" t="inlineStr"/>
+      <c r="AB184" t="inlineStr"/>
+      <c r="AC184" t="inlineStr"/>
+      <c r="AD184" t="inlineStr"/>
+      <c r="AE184" t="inlineStr"/>
+      <c r="AF184" t="inlineStr"/>
+      <c r="AG184" t="inlineStr"/>
+      <c r="AH184" t="inlineStr"/>
+      <c r="AI184" t="inlineStr"/>
+      <c r="AJ184" t="inlineStr"/>
+      <c r="AK184" t="inlineStr"/>
+      <c r="AL184" t="inlineStr"/>
+      <c r="AM184" t="inlineStr"/>
+      <c r="AN184" t="inlineStr"/>
+      <c r="AO184" t="inlineStr"/>
+      <c r="AP184" t="inlineStr"/>
+      <c r="AQ184" t="inlineStr"/>
+      <c r="AR184" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS184" t="n">
+        <v>20</v>
+      </c>
+      <c r="AT184" t="n">
+        <v>130</v>
+      </c>
+      <c r="AU184" t="inlineStr"/>
+      <c r="AV184" t="inlineStr"/>
+      <c r="AW184" t="inlineStr"/>
+      <c r="AX184" t="inlineStr"/>
+      <c r="AY184" t="inlineStr"/>
+      <c r="AZ184" t="inlineStr"/>
+      <c r="BA184" t="inlineStr"/>
+      <c r="BB184" t="inlineStr"/>
+      <c r="BC184" t="inlineStr"/>
+      <c r="BD184" t="inlineStr"/>
+      <c r="BE184" t="inlineStr"/>
+      <c r="BF184" t="inlineStr"/>
+      <c r="BG184" t="inlineStr"/>
+      <c r="BH184" t="inlineStr"/>
+      <c r="BI184" t="inlineStr"/>
+      <c r="BJ184" t="inlineStr"/>
+      <c r="BK184" t="inlineStr"/>
+      <c r="BL184" t="inlineStr"/>
+      <c r="BM184" t="inlineStr"/>
+      <c r="BN184" t="inlineStr"/>
+      <c r="BO184" t="inlineStr"/>
+      <c r="BP184" t="inlineStr"/>
+      <c r="BQ184" t="inlineStr"/>
+      <c r="BR184" t="inlineStr"/>
+      <c r="BS184" t="inlineStr"/>
+      <c r="BT184" t="inlineStr"/>
+      <c r="BU184" t="inlineStr"/>
+      <c r="BV184" t="inlineStr"/>
+      <c r="BW184" t="inlineStr"/>
+      <c r="BX184" t="inlineStr"/>
+      <c r="BY184" t="inlineStr"/>
+      <c r="BZ184" t="inlineStr"/>
+      <c r="CA184" t="inlineStr"/>
+      <c r="CB184" t="inlineStr"/>
+      <c r="CC184" t="inlineStr"/>
+      <c r="CD184" t="inlineStr"/>
+      <c r="CE184" t="inlineStr"/>
+      <c r="CF184" t="inlineStr"/>
+      <c r="CG184" t="inlineStr"/>
+      <c r="CH184" t="inlineStr"/>
+      <c r="CI184" t="inlineStr"/>
+      <c r="CJ184" t="inlineStr"/>
+      <c r="CK184" t="inlineStr"/>
+      <c r="CL184" t="inlineStr"/>
+      <c r="CM184" t="inlineStr"/>
+      <c r="CN184" t="inlineStr"/>
+      <c r="CO184" t="inlineStr"/>
+      <c r="CP184" t="inlineStr"/>
+      <c r="CQ184" t="inlineStr"/>
+      <c r="CR184" t="inlineStr"/>
+      <c r="CS184" t="inlineStr"/>
+      <c r="CT184" t="inlineStr"/>
+      <c r="CU184" t="inlineStr"/>
+      <c r="CV184" t="inlineStr"/>
+      <c r="CW184" t="inlineStr"/>
+      <c r="CX184" t="inlineStr"/>
+      <c r="CY184" t="inlineStr"/>
+      <c r="CZ184" t="inlineStr"/>
+      <c r="DA184" t="inlineStr"/>
+      <c r="DB184" t="inlineStr"/>
+      <c r="DC184" t="inlineStr"/>
+      <c r="DD184" t="inlineStr"/>
+      <c r="DE184" t="inlineStr"/>
+      <c r="DF184" t="inlineStr"/>
+      <c r="DG184" t="inlineStr"/>
+      <c r="DH184" t="inlineStr"/>
+      <c r="DI184" t="inlineStr"/>
+      <c r="DJ184" t="inlineStr"/>
+      <c r="DK184" t="inlineStr"/>
+      <c r="DL184" t="inlineStr"/>
+      <c r="DM184" t="inlineStr"/>
+      <c r="DN184" t="inlineStr"/>
+      <c r="DO184" t="inlineStr"/>
+      <c r="DP184" t="inlineStr"/>
+      <c r="DQ184" t="inlineStr"/>
+      <c r="DR184" t="inlineStr"/>
+      <c r="DS184" t="inlineStr"/>
+      <c r="DT184" t="inlineStr"/>
+      <c r="DU184" t="inlineStr"/>
+      <c r="DV184" t="inlineStr"/>
+      <c r="DW184" t="inlineStr"/>
+      <c r="DX184" t="inlineStr"/>
+      <c r="DY184" t="inlineStr"/>
+      <c r="DZ184" t="inlineStr"/>
+      <c r="EA184" t="inlineStr"/>
+      <c r="EB184" t="inlineStr"/>
+      <c r="EC184" t="inlineStr"/>
+      <c r="ED184" t="n">
+        <v>2</v>
+      </c>
+      <c r="EE184" t="n">
+        <v>4</v>
+      </c>
+      <c r="EF184" t="n">
+        <v>128.09</v>
+      </c>
+      <c r="EG184" t="inlineStr"/>
+      <c r="EH184" t="inlineStr"/>
+      <c r="EI184" t="inlineStr"/>
+      <c r="EJ184" t="inlineStr"/>
+      <c r="EK184" t="inlineStr"/>
+      <c r="EL184" t="inlineStr"/>
+      <c r="EM184" t="inlineStr"/>
+      <c r="EN184" t="inlineStr"/>
+      <c r="EO184" t="inlineStr"/>
+      <c r="EP184" t="inlineStr"/>
+      <c r="EQ184" t="inlineStr"/>
+      <c r="ER184" t="inlineStr"/>
+      <c r="ES184" t="inlineStr"/>
+      <c r="ET184" t="inlineStr"/>
+      <c r="EU184" t="inlineStr"/>
+      <c r="EV184" t="inlineStr"/>
+      <c r="EW184" t="inlineStr"/>
+      <c r="EX184" t="inlineStr"/>
+      <c r="EY184" t="inlineStr"/>
+      <c r="EZ184" t="inlineStr"/>
+      <c r="FA184" t="inlineStr"/>
+      <c r="FB184" t="inlineStr"/>
+      <c r="FC184" t="inlineStr"/>
+      <c r="FD184" t="inlineStr"/>
+      <c r="FE184" t="inlineStr"/>
+      <c r="FF184" t="inlineStr"/>
+      <c r="FG184" t="inlineStr"/>
+      <c r="FH184" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="FI184" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="FJ184" t="n">
         <v>0</v>
       </c>
-      <c r="GW181" t="n">
+      <c r="FK184" t="inlineStr">
+        <is>
+          <t>Pequi (Caryocar brasiliense)</t>
+        </is>
+      </c>
+      <c r="FL184" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="FM184" t="n">
+        <v>10</v>
+      </c>
+      <c r="FN184" t="n">
+        <v>20</v>
+      </c>
+      <c r="FO184" t="n">
+        <v>900</v>
+      </c>
+      <c r="FP184" t="inlineStr"/>
+      <c r="FQ184" t="inlineStr"/>
+      <c r="FR184" t="inlineStr"/>
+      <c r="FS184" t="inlineStr"/>
+      <c r="FT184" t="inlineStr"/>
+      <c r="FU184" t="inlineStr"/>
+      <c r="FV184" t="inlineStr"/>
+      <c r="FW184" t="inlineStr"/>
+      <c r="FX184" t="inlineStr"/>
+      <c r="FY184" t="inlineStr"/>
+      <c r="FZ184" t="inlineStr"/>
+      <c r="GA184" t="inlineStr"/>
+      <c r="GB184" t="inlineStr"/>
+      <c r="GC184" t="inlineStr"/>
+      <c r="GD184" t="inlineStr"/>
+      <c r="GE184" t="inlineStr"/>
+      <c r="GF184" t="inlineStr"/>
+      <c r="GG184" t="inlineStr"/>
+      <c r="GH184" t="inlineStr"/>
+      <c r="GI184" t="inlineStr"/>
+      <c r="GJ184" t="inlineStr"/>
+      <c r="GK184" t="inlineStr"/>
+      <c r="GL184" t="inlineStr"/>
+      <c r="GM184" t="inlineStr"/>
+      <c r="GN184" t="inlineStr"/>
+      <c r="GO184" t="inlineStr"/>
+      <c r="GP184" t="inlineStr"/>
+      <c r="GQ184" t="n">
         <v>0</v>
       </c>
-      <c r="GX181" t="n">
+      <c r="GR184" t="inlineStr"/>
+      <c r="GS184" t="n">
         <v>0</v>
       </c>
-      <c r="GY181" t="inlineStr"/>
-      <c r="GZ181" t="n">
+      <c r="GT184" t="n">
         <v>0</v>
       </c>
-      <c r="HA181" t="n">
+      <c r="GU184" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV184" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW184" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX184" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY184" t="inlineStr"/>
+      <c r="GZ184" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA184" t="n">
         <v>12.6</v>
       </c>
-      <c r="HB181" t="n">
+      <c r="HB184" t="n">
         <v>77.2</v>
       </c>
-      <c r="HC181" t="n">
+      <c r="HC184" t="n">
         <v>10.2</v>
       </c>
-      <c r="HD181" t="n">
+      <c r="HD184" t="n">
         <v>0</v>
       </c>
-      <c r="HE181" t="n">
+      <c r="HE184" t="n">
         <v>0</v>
       </c>
-      <c r="HF181" t="n">
+      <c r="HF184" t="n">
         <v>0</v>
       </c>
-      <c r="HG181" t="n">
+      <c r="HG184" t="n">
         <v>0</v>
       </c>
-      <c r="HH181" t="n">
+      <c r="HH184" t="n">
         <v>0</v>
       </c>
-      <c r="HI181" t="n">
+      <c r="HI184" t="n">
         <v>0</v>
       </c>
-      <c r="HJ181" t="n">
+      <c r="HJ184" t="n">
         <v>0</v>
       </c>
-      <c r="HK181" t="n">
+      <c r="HK184" t="n">
         <v>0</v>
       </c>
-      <c r="HL181" t="n">
+      <c r="HL184" t="n">
         <v>0</v>
       </c>
-      <c r="HM181" t="n">
+      <c r="HM184" t="n">
         <v>0</v>
       </c>
-      <c r="HN181" t="n">
+      <c r="HN184" t="n">
         <v>100</v>
       </c>
-      <c r="HO181" t="n">
+      <c r="HO184" t="n">
         <v>0</v>
       </c>
-      <c r="HP181" t="n">
+      <c r="HP184" t="n">
         <v>100</v>
       </c>
-      <c r="HQ181" t="n">
+      <c r="HQ184" t="n">
         <v>0</v>
       </c>
-      <c r="HR181" t="n">
+      <c r="HR184" t="n">
         <v>44.03</v>
       </c>
-      <c r="HS181" t="n">
+      <c r="HS184" t="n">
         <v>39.06</v>
       </c>
-      <c r="HT181" t="n">
+      <c r="HT184" t="n">
         <v>0</v>
       </c>
-      <c r="HU181" t="n">
+      <c r="HU184" t="n">
         <v>0</v>
       </c>
-      <c r="HV181" t="n">
+      <c r="HV184" t="n">
         <v>0</v>
       </c>
-      <c r="HW181" t="n">
+      <c r="HW184" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace Samuel Kimenyi spreadsheet with revised maintenance data.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Consultants Data Validation - Master Database.xlsx
+++ b/Consultants Data Validation - Master Database.xlsx
@@ -53998,7 +53998,7 @@
         <v>2</v>
       </c>
       <c r="O178" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="P178" t="n">
         <v>100</v>
@@ -54094,10 +54094,10 @@
         <v>2</v>
       </c>
       <c r="DA178" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="DB178" t="n">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="DC178" t="inlineStr"/>
       <c r="DD178" t="inlineStr"/>
@@ -54133,7 +54133,7 @@
         <v>20</v>
       </c>
       <c r="EF178" t="n">
-        <v>220</v>
+        <v>100</v>
       </c>
       <c r="EG178" t="inlineStr"/>
       <c r="EH178" t="inlineStr"/>
@@ -54395,7 +54395,7 @@
         <v>2</v>
       </c>
       <c r="AS179" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AT179" t="n">
         <v>163</v>
@@ -54467,10 +54467,10 @@
         <v>2</v>
       </c>
       <c r="DA179" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="DB179" t="n">
-        <v>450</v>
+        <v>110</v>
       </c>
       <c r="DC179" t="inlineStr"/>
       <c r="DD179" t="inlineStr"/>
@@ -54506,7 +54506,7 @@
         <v>20</v>
       </c>
       <c r="EF179" t="n">
-        <v>390</v>
+        <v>180</v>
       </c>
       <c r="EG179" t="inlineStr"/>
       <c r="EH179" t="inlineStr"/>
@@ -54768,7 +54768,7 @@
         <v>2</v>
       </c>
       <c r="O180" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="P180" t="n">
         <v>70</v>
@@ -54864,10 +54864,10 @@
         <v>2</v>
       </c>
       <c r="DA180" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="DB180" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="DC180" t="inlineStr"/>
       <c r="DD180" t="inlineStr"/>
@@ -54903,7 +54903,7 @@
         <v>20</v>
       </c>
       <c r="EF180" t="n">
-        <v>190</v>
+        <v>110</v>
       </c>
       <c r="EG180" t="inlineStr"/>
       <c r="EH180" t="inlineStr"/>
@@ -55165,10 +55165,10 @@
         <v>2</v>
       </c>
       <c r="AS181" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="AT181" t="n">
-        <v>165</v>
+        <v>100</v>
       </c>
       <c r="AU181" t="inlineStr"/>
       <c r="AV181" t="inlineStr"/>
@@ -55237,10 +55237,10 @@
         <v>2</v>
       </c>
       <c r="DA181" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="DB181" t="n">
-        <v>220</v>
+        <v>100</v>
       </c>
       <c r="DC181" t="inlineStr"/>
       <c r="DD181" t="inlineStr"/>
@@ -55273,10 +55273,10 @@
         <v>2</v>
       </c>
       <c r="EE181" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="EF181" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="EG181" t="inlineStr"/>
       <c r="EH181" t="inlineStr"/>
@@ -55538,10 +55538,10 @@
         <v>2</v>
       </c>
       <c r="O182" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="P182" t="n">
-        <v>245</v>
+        <v>150</v>
       </c>
       <c r="Q182" t="inlineStr"/>
       <c r="R182" t="inlineStr"/>
@@ -55634,10 +55634,10 @@
         <v>2</v>
       </c>
       <c r="DA182" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="DB182" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="DC182" t="inlineStr"/>
       <c r="DD182" t="inlineStr"/>
@@ -55673,7 +55673,7 @@
         <v>20</v>
       </c>
       <c r="EF182" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="EG182" t="inlineStr"/>
       <c r="EH182" t="inlineStr"/>
@@ -55935,7 +55935,7 @@
         <v>2</v>
       </c>
       <c r="AS183" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="AT183" t="n">
         <v>260</v>
@@ -56007,10 +56007,10 @@
         <v>2</v>
       </c>
       <c r="DA183" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="DB183" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="DC183" t="inlineStr"/>
       <c r="DD183" t="inlineStr"/>
@@ -56043,10 +56043,10 @@
         <v>2</v>
       </c>
       <c r="EE183" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="EF183" t="n">
-        <v>330</v>
+        <v>210</v>
       </c>
       <c r="EG183" t="inlineStr"/>
       <c r="EH183" t="inlineStr"/>

</xml_diff>